<commit_message>
Refactored database schema and SQL views to include proficiency levels for skills and tools at smarter place; update master database and finally executed pipeline.
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/02_Data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FDBC784-BA71-A04D-8403-FDB16679588B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2525185F-5315-E947-981A-B32C83E1325B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25580" yWindow="600" windowWidth="25620" windowHeight="28200" firstSheet="7" activeTab="13" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28500" windowHeight="28200" firstSheet="1" activeTab="6" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
     <sheet name="person_tools" sheetId="9" r:id="rId13"/>
     <sheet name="portfolio_tools" sheetId="7" r:id="rId14"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="297">
   <si>
     <t>Graduation</t>
   </si>
@@ -177,12 +177,6 @@
     <t>Characterization of floc-forming, fast-sedimenting microalgae-bacteria consortia used for low-cost biomass harvesting in chemostatic bioreactors</t>
   </si>
   <si>
-    <t>https://doi.org/10.21203/rs.3.rs-6327003/v1</t>
-  </si>
-  <si>
-    <t>Physiologic manipulation of microalgae-bacteria consortia: chances and limitations</t>
-  </si>
-  <si>
     <t>Biofilm-driven flocculation in microalgae-bacteria consortia: Mechanisms and biotechnological implications</t>
   </si>
   <si>
@@ -240,15 +234,6 @@
     <t>Investigation of enzymes involved in pyrrolizidine alkaloid biosynthesis using the hairy root system</t>
   </si>
   <si>
-    <t>Paper I</t>
-  </si>
-  <si>
-    <t>Paper II</t>
-  </si>
-  <si>
-    <t>Paper III</t>
-  </si>
-  <si>
     <t>Dashboard visualising PhD thesis data</t>
   </si>
   <si>
@@ -411,18 +396,6 @@
     <t>domain_id</t>
   </si>
   <si>
-    <t>Here i learned</t>
-  </si>
-  <si>
-    <t>Here I developed</t>
-  </si>
-  <si>
-    <t>Here I Teached</t>
-  </si>
-  <si>
-    <t>Here I don't know</t>
-  </si>
-  <si>
     <t>activity_id</t>
   </si>
   <si>
@@ -450,12 +423,6 @@
     <t>Funding Consultant</t>
   </si>
   <si>
-    <t>My journey into data science taught me how to translate raw data into actionable insights. From statistical modeling to visualization, I learned how to use various tools. Combining technical skills with storytelling allows me to uncover patterns, support decisions and communicate results effectively.</t>
-  </si>
-  <si>
-    <t>Working with SMEs and research institutions taught me how to navigate funding landscapes and bring together different partners to work towards shared goals. I developed strategic innovation skills, learned to transform ideas into structured projects and shaped R&amp;D networks that drive progressive technologies.</t>
-  </si>
-  <si>
     <t>I thrive at the intersection of science, innovation and data. My path taught me to adapt quickly, communicate effectively and create impact in diverse contexts. Along the way, I learned to shape projects strategically and make complex information accessible through clear visualization and storytelling.</t>
   </si>
   <si>
@@ -495,9 +462,6 @@
     <t>certificate_id</t>
   </si>
   <si>
-    <t>https://public.tableau.com/app/profile/cedric.hering.peter/viz/CV-Dashboard_17551211549430/Resume_0_4?publish=yes</t>
-  </si>
-  <si>
     <t>status</t>
   </si>
   <si>
@@ -585,9 +549,6 @@
     <t>#Science #Microalgae #Sustainability</t>
   </si>
   <si>
-    <t>Through academic research, I learned to explore complex biological systems with creativity and persistence. Investigating microorganismic interactions sharpened my skills in problem-solving, experimental design and data analysis  - insights that I now apply beyond the lab to innovation and sustainability.</t>
-  </si>
-  <si>
     <t>hashtags</t>
   </si>
   <si>
@@ -937,6 +898,48 @@
   </si>
   <si>
     <t>ZIM-Network for    Bioeconomy</t>
+  </si>
+  <si>
+    <t>Processed and analyzed large biological datasets. Designed reproducible data workflows and scientific models using Python (statistical analysis, multivariate techniques). Published results in peer-reviewed journals.</t>
+  </si>
+  <si>
+    <t>Advised clients on innovation strategies and technology-driven projects, including AI and data-related applications (from idea framing to successful funding acquisition). Collaborated with cross-functional stake-holders across industry &amp; research.</t>
+  </si>
+  <si>
+    <t>Explored a complex phototropic system which is used for sustainable bioremediation (water cleaning) through academic biotechnological research. Sharpened skills in problem-solving, experimental design and data analysis. Published results in peer-reviewed journals.</t>
+  </si>
+  <si>
+    <t>As a hobby, I create games focusing on model creation (Blender) and engine coding (Unity).</t>
+  </si>
+  <si>
+    <t>As a lecturer, I gave students insights into the field of general molecular biology.</t>
+  </si>
+  <si>
+    <t>After graduation, I specialist into the field of biology. Explored the beauty and detailness of animals, plants and microorganisms.</t>
+  </si>
+  <si>
+    <t>Physiological responses of floc-forming microalgae-bacteria consortia to environmental perturbations</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1007/s10811-026-03813-z</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.algal.2026.104660</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/showcase/zim-innovationsnetzwerk-bluepathways/about/</t>
+  </si>
+  <si>
+    <t>https://public.tableau.com/app/profile/cedric.hering.peter/viz/CV-Dashboard_17551211549430/Published_Apr-26?publish=yes</t>
+  </si>
+  <si>
+    <t>Paper in Bioresource Technology</t>
+  </si>
+  <si>
+    <t>Paper in Journal  of Applied Phycology</t>
+  </si>
+  <si>
+    <t>Paper in Algal    Research</t>
   </si>
 </sst>
 </file>
@@ -1091,15 +1094,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color theme="4" tint="0.39997558519241921"/>
       </left>
@@ -1145,13 +1139,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1167,32 +1172,49 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="11">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -1289,12 +1311,6 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1341,6 +1357,12 @@
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1365,19 +1387,18 @@
     <tableColumn id="6" xr3:uid="{08E97EF2-2A58-9142-81F6-5F4A1B6CAF2C}" name="city"/>
     <tableColumn id="5" xr3:uid="{831CB986-42F5-9D46-860A-8100DBA32197}" name="province"/>
     <tableColumn id="4" xr3:uid="{7564C2FC-BB92-7742-A00C-C96E922B28EF}" name="country"/>
-    <tableColumn id="9" xr3:uid="{C61E8E18-A34B-F64D-911A-EB79E1C91129}" name="birth_date" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{C61E8E18-A34B-F64D-911A-EB79E1C91129}" name="birth_date" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{8AD25C77-43E5-DB4D-BFBA-E3C97FDA744F}" name="Table913" displayName="Table913" ref="A1:C25" totalsRowShown="0">
-  <autoFilter ref="A1:C25" xr:uid="{CF8F687B-EE5F-C44C-BC54-A0EBA7BD1D0F}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{8AD25C77-43E5-DB4D-BFBA-E3C97FDA744F}" name="Table913" displayName="Table913" ref="A1:B25" totalsRowShown="0">
+  <autoFilter ref="A1:B25" xr:uid="{CF8F687B-EE5F-C44C-BC54-A0EBA7BD1D0F}"/>
+  <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{33A0361B-07E2-FF48-8CB7-DC3C9AC56FB2}" name="person_id"/>
     <tableColumn id="2" xr3:uid="{A6316854-AD5D-7F41-98D4-16938B4ECC90}" name="skill_id"/>
-    <tableColumn id="3" xr3:uid="{8D6F357B-B5DC-614D-ADE1-FC796A9BF0A6}" name="proficiency_level"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1395,9 +1416,9 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D4D9EF09-F165-3445-9DF8-3380B4CE8578}" name="Table4" displayName="Table4" ref="A1:E35" totalsRowShown="0">
-  <autoFilter ref="A1:E35" xr:uid="{D4D9EF09-F165-3445-9DF8-3380B4CE8578}">
-    <filterColumn colId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D4D9EF09-F165-3445-9DF8-3380B4CE8578}" name="Table4" displayName="Table4" ref="A1:F35" totalsRowShown="0">
+  <autoFilter ref="A1:F35" xr:uid="{D4D9EF09-F165-3445-9DF8-3380B4CE8578}">
+    <filterColumn colId="5">
       <filters>
         <filter val="1"/>
         <filter val="13"/>
@@ -1409,13 +1430,14 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E35">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F35">
     <sortCondition ref="A1:A35"/>
   </sortState>
-  <tableColumns count="5">
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9322AF04-06A6-7A4B-ADE9-7C818778F408}" name="tool_id"/>
     <tableColumn id="2" xr3:uid="{ED109F91-6525-6041-8EBB-023043C5731A}" name="name"/>
     <tableColumn id="3" xr3:uid="{A9ED79A6-606F-3B49-B27A-CA6E23786847}" name="category"/>
+    <tableColumn id="7" xr3:uid="{379B4B50-0DFF-B146-9CED-6E18F96B753E}" name="proficiency_level"/>
     <tableColumn id="5" xr3:uid="{43A488CD-EE4E-D84D-A416-730D5ACBD468}" name="description"/>
     <tableColumn id="4" xr3:uid="{1F96A067-5F7F-9944-B83D-DAD6F8490299}" name="project occurance">
       <calculatedColumnFormula>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</calculatedColumnFormula>
@@ -1426,12 +1448,11 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{CF8F687B-EE5F-C44C-BC54-A0EBA7BD1D0F}" name="Table9" displayName="Table9" ref="A1:C35" totalsRowShown="0">
-  <autoFilter ref="A1:C35" xr:uid="{CF8F687B-EE5F-C44C-BC54-A0EBA7BD1D0F}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{CF8F687B-EE5F-C44C-BC54-A0EBA7BD1D0F}" name="Table9" displayName="Table9" ref="A1:B35" totalsRowShown="0">
+  <autoFilter ref="A1:B35" xr:uid="{CF8F687B-EE5F-C44C-BC54-A0EBA7BD1D0F}"/>
+  <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{36CA1518-31C3-2C4E-9E65-D2E62113B101}" name="person_id"/>
     <tableColumn id="2" xr3:uid="{7163B45B-BAF7-A149-BBD9-D86966F3B602}" name="tool_id"/>
-    <tableColumn id="3" xr3:uid="{C0077BFF-F346-F345-8BB5-F97A4473DF6C}" name="proficiency_level"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1474,8 +1495,8 @@
     <tableColumn id="3" xr3:uid="{519CB3FD-482A-2B44-9C5A-9E797E3F98E4}" name="title"/>
     <tableColumn id="4" xr3:uid="{0DBFEBFC-D18A-6F4E-87F2-C8D4D16C7E2D}" name="organization"/>
     <tableColumn id="9" xr3:uid="{3E657E01-C34B-0B41-8B45-85D9AE50305B}" name="location"/>
-    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="6"/>
     <tableColumn id="8" xr3:uid="{4B60B559-FFE2-0449-BD87-E423F2579CE2}" name="description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1486,7 +1507,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}" name="Table14" displayName="Table14" ref="A1:B24" totalsRowShown="0">
   <autoFilter ref="A1:B24" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{647E29E8-3B30-6747-952B-856B15C586DD}" name="domain_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1527,8 +1548,8 @@
     <tableColumn id="6" xr3:uid="{D37906CD-C2EB-8A40-AA51-891ADDD2F0F3}" name="person_id"/>
     <tableColumn id="8" xr3:uid="{912FC1CE-8929-A840-BCE1-17117B008FD3}" name="title"/>
     <tableColumn id="11" xr3:uid="{8675359A-ECB9-7944-B6E4-F8EFBA93E841}" name="description"/>
-    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="10"/>
+    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="9"/>
     <tableColumn id="1" xr3:uid="{D859FDAD-79F9-EC41-ACD6-64B4107CA00A}" name="status"/>
     <tableColumn id="12" xr3:uid="{267EBF1D-F600-6746-8520-55E6EE075513}" name="link"/>
   </tableColumns>
@@ -1548,15 +1569,16 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{7F565E25-C764-3143-AFFA-BCE408907871}" name="Table412" displayName="Table412" ref="A1:E25" totalsRowShown="0">
-  <autoFilter ref="A1:E25" xr:uid="{D4D9EF09-F165-3445-9DF8-3380B4CE8578}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{7F565E25-C764-3143-AFFA-BCE408907871}" name="Table412" displayName="Table412" ref="A1:F25" totalsRowShown="0">
+  <autoFilter ref="A1:F25" xr:uid="{D4D9EF09-F165-3445-9DF8-3380B4CE8578}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F25">
     <sortCondition ref="A1:A25"/>
   </sortState>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{DC3EED09-C75A-A540-B993-B2129AB8E714}" name="skill_id" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{42FD44F0-B09F-0547-A986-21BFB4182840}" name="name" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{210EF8DD-2CB7-914A-90FE-26900DEF4416}" name="category" dataDxfId="1"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{DC3EED09-C75A-A540-B993-B2129AB8E714}" name="skill_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{42FD44F0-B09F-0547-A986-21BFB4182840}" name="name" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{210EF8DD-2CB7-914A-90FE-26900DEF4416}" name="category" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{F5C94330-B6D8-C140-A633-2F241C9BBCC6}" name="proficiency_level" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{D6C18DDB-3DCD-4744-94D9-9336C79C3BDE}" name="description"/>
     <tableColumn id="5" xr3:uid="{3D69894F-FAB2-F24C-B720-564E0EBF08D7}" name="project occurance" dataDxfId="0">
       <calculatedColumnFormula>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</calculatedColumnFormula>
@@ -1885,7 +1907,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA051E34-3D1F-4D4A-8D3B-9B3E0598856B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
@@ -1900,28 +1922,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H1" t="s">
         <v>94</v>
-      </c>
-      <c r="B1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E1" t="s">
-        <v>140</v>
-      </c>
-      <c r="F1" t="s">
-        <v>138</v>
-      </c>
-      <c r="G1" t="s">
-        <v>139</v>
-      </c>
-      <c r="H1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -1929,22 +1951,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E2" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="F2" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="G2" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="H2" s="4">
         <v>34220</v>
@@ -1962,300 +1984,224 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4F44A1C-67CC-0446-A21E-A9C26D83AD6C}">
   <sheetPr codeName="Sheet12"/>
-  <dimension ref="A1:J25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14.1640625" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C1" t="s">
-        <v>108</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="C1" s="9"/>
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
       <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
-      <c r="C3">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
-      <c r="C7">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
-      <c r="C8">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
-      <c r="C9">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1</v>
       </c>
       <c r="B10">
         <v>9</v>
       </c>
-      <c r="C10">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>1</v>
       </c>
       <c r="B11">
         <v>10</v>
       </c>
-      <c r="C11">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1</v>
       </c>
       <c r="B12">
         <v>11</v>
       </c>
-      <c r="C12">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1</v>
       </c>
       <c r="B13">
         <v>12</v>
       </c>
-      <c r="C13">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1</v>
       </c>
       <c r="B14">
         <v>13</v>
       </c>
-      <c r="C14">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1</v>
       </c>
       <c r="B15">
         <v>14</v>
       </c>
-      <c r="C15">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1</v>
       </c>
       <c r="B16">
         <v>15</v>
       </c>
-      <c r="C16">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>1</v>
       </c>
       <c r="B17">
         <v>16</v>
       </c>
-      <c r="C17">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>1</v>
       </c>
       <c r="B18">
         <v>17</v>
       </c>
-      <c r="C18">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1</v>
       </c>
       <c r="B19">
         <v>18</v>
       </c>
-      <c r="C19">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1</v>
       </c>
       <c r="B20">
         <v>19</v>
       </c>
-      <c r="C20">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1</v>
       </c>
       <c r="B21">
         <v>20</v>
       </c>
-      <c r="C21">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>1</v>
       </c>
       <c r="B22">
         <v>21</v>
       </c>
-      <c r="C22">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>1</v>
       </c>
       <c r="B23">
         <v>22</v>
       </c>
-      <c r="C23">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>1</v>
       </c>
       <c r="B24">
         <v>23</v>
       </c>
-      <c r="C24">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>1</v>
       </c>
       <c r="B25">
         <v>24</v>
-      </c>
-      <c r="C25">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2270,7 +2216,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C6AC091-0337-EE42-81A2-CB3A7445D977}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:B156"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.83203125" bestFit="1" customWidth="1"/>
@@ -2278,10 +2224,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -3535,40 +3481,44 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FF6DBFF-8203-BA44-A62E-5965AC08ED0E}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:I52"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="31.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="59.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="59.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B1" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D1" t="s">
         <v>103</v>
       </c>
-      <c r="E1" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="F1" s="9"/>
+      <c r="E1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>241</v>
+      </c>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
       <c r="I1" s="9"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1" s="9"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3576,17 +3526,20 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D2" t="s">
-        <v>193</v>
-      </c>
-      <c r="E2">
+        <v>173</v>
+      </c>
+      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>180</v>
+      </c>
+      <c r="F2">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3594,53 +3547,62 @@
         <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>186</v>
-      </c>
-      <c r="D3" t="s">
-        <v>192</v>
-      </c>
-      <c r="E3">
+        <v>173</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>179</v>
+      </c>
+      <c r="F3">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="C4" t="s">
-        <v>186</v>
-      </c>
-      <c r="D4" t="s">
-        <v>194</v>
-      </c>
-      <c r="E4">
+        <v>173</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>181</v>
+      </c>
+      <c r="F4">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="C5" t="s">
-        <v>186</v>
-      </c>
-      <c r="D5" t="s">
-        <v>194</v>
-      </c>
-      <c r="E5">
+        <v>173</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+      <c r="E5" t="s">
+        <v>181</v>
+      </c>
+      <c r="F5">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3648,17 +3610,20 @@
         <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>186</v>
-      </c>
-      <c r="D6" t="s">
-        <v>195</v>
-      </c>
-      <c r="E6">
+        <v>173</v>
+      </c>
+      <c r="D6">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>182</v>
+      </c>
+      <c r="F6">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3666,17 +3631,20 @@
         <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>186</v>
-      </c>
-      <c r="D7" t="s">
-        <v>196</v>
-      </c>
-      <c r="E7">
+        <v>173</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>183</v>
+      </c>
+      <c r="F7">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3684,35 +3652,41 @@
         <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>186</v>
-      </c>
-      <c r="D8" t="s">
-        <v>197</v>
-      </c>
-      <c r="E8">
+        <v>173</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>184</v>
+      </c>
+      <c r="F8">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>186</v>
-      </c>
-      <c r="D9" t="s">
-        <v>201</v>
-      </c>
-      <c r="E9">
+        <v>173</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>188</v>
+      </c>
+      <c r="F9">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3720,71 +3694,83 @@
         <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>186</v>
-      </c>
-      <c r="D10" t="s">
-        <v>198</v>
-      </c>
-      <c r="E10">
+        <v>173</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>185</v>
+      </c>
+      <c r="F10">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>180</v>
-      </c>
-      <c r="D11" t="s">
-        <v>199</v>
-      </c>
-      <c r="E11">
+        <v>167</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>186</v>
+      </c>
+      <c r="F11">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>180</v>
-      </c>
-      <c r="D12" t="s">
-        <v>200</v>
-      </c>
-      <c r="E12">
+        <v>167</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>187</v>
+      </c>
+      <c r="F12">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>292</v>
+        <v>279</v>
       </c>
       <c r="C13" t="s">
-        <v>185</v>
-      </c>
-      <c r="D13" t="s">
-        <v>202</v>
-      </c>
-      <c r="E13">
+        <v>172</v>
+      </c>
+      <c r="D13">
+        <v>5</v>
+      </c>
+      <c r="E13" t="s">
+        <v>189</v>
+      </c>
+      <c r="F13">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3792,71 +3778,83 @@
         <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>186</v>
-      </c>
-      <c r="D14" t="s">
-        <v>293</v>
-      </c>
-      <c r="E14">
+        <v>173</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="E14" t="s">
+        <v>280</v>
+      </c>
+      <c r="F14">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C15" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15" t="s">
-        <v>205</v>
-      </c>
-      <c r="E15">
+        <v>75</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15" t="s">
+        <v>192</v>
+      </c>
+      <c r="F15">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>80</v>
-      </c>
-      <c r="D16" t="s">
-        <v>205</v>
-      </c>
-      <c r="E16">
+        <v>75</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>192</v>
+      </c>
+      <c r="F16">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>80</v>
-      </c>
-      <c r="D17" t="s">
-        <v>206</v>
-      </c>
-      <c r="E17">
+        <v>75</v>
+      </c>
+      <c r="D17">
+        <v>3</v>
+      </c>
+      <c r="E17" t="s">
+        <v>193</v>
+      </c>
+      <c r="F17">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3864,345 +3862,407 @@
         <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>186</v>
-      </c>
-      <c r="D18" t="s">
-        <v>207</v>
-      </c>
-      <c r="E18">
+        <v>173</v>
+      </c>
+      <c r="D18">
+        <v>3</v>
+      </c>
+      <c r="E18" t="s">
+        <v>194</v>
+      </c>
+      <c r="F18">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>290</v>
+        <v>277</v>
       </c>
       <c r="C19" t="s">
-        <v>185</v>
-      </c>
-      <c r="D19" t="s">
-        <v>210</v>
-      </c>
-      <c r="E19">
+        <v>172</v>
+      </c>
+      <c r="D19">
+        <v>4</v>
+      </c>
+      <c r="E19" t="s">
+        <v>197</v>
+      </c>
+      <c r="F19">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C20" t="s">
-        <v>185</v>
-      </c>
-      <c r="D20" t="s">
-        <v>212</v>
-      </c>
-      <c r="E20">
+        <v>172</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20" t="s">
+        <v>199</v>
+      </c>
+      <c r="F20">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C21" t="s">
-        <v>185</v>
-      </c>
-      <c r="D21" t="s">
-        <v>211</v>
-      </c>
-      <c r="E21">
+        <v>172</v>
+      </c>
+      <c r="D21">
+        <v>3</v>
+      </c>
+      <c r="E21" t="s">
+        <v>198</v>
+      </c>
+      <c r="F21">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" s="17" t="s">
-        <v>90</v>
+      <c r="B22" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="D22" t="s">
-        <v>213</v>
-      </c>
-      <c r="E22">
+        <v>78</v>
+      </c>
+      <c r="D22">
+        <v>5</v>
+      </c>
+      <c r="E22" t="s">
+        <v>200</v>
+      </c>
+      <c r="F22">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>83</v>
-      </c>
-      <c r="D23" t="s">
-        <v>214</v>
-      </c>
-      <c r="E23">
+        <v>78</v>
+      </c>
+      <c r="D23">
+        <v>4</v>
+      </c>
+      <c r="E23" t="s">
+        <v>201</v>
+      </c>
+      <c r="F23">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>83</v>
-      </c>
-      <c r="D24" t="s">
-        <v>215</v>
-      </c>
-      <c r="E24">
+        <v>78</v>
+      </c>
+      <c r="D24">
+        <v>2</v>
+      </c>
+      <c r="E24" t="s">
+        <v>202</v>
+      </c>
+      <c r="F24">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C25" t="s">
-        <v>83</v>
-      </c>
-      <c r="D25" t="s">
-        <v>216</v>
-      </c>
-      <c r="E25">
+        <v>78</v>
+      </c>
+      <c r="D25">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>203</v>
+      </c>
+      <c r="F25">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>219</v>
+        <v>206</v>
       </c>
       <c r="C26" t="s">
-        <v>83</v>
-      </c>
-      <c r="D26" t="s">
-        <v>217</v>
-      </c>
-      <c r="E26">
+        <v>78</v>
+      </c>
+      <c r="D26">
+        <v>5</v>
+      </c>
+      <c r="E26" t="s">
+        <v>204</v>
+      </c>
+      <c r="F26">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="C27" t="s">
-        <v>83</v>
-      </c>
-      <c r="D27" t="s">
-        <v>220</v>
-      </c>
-      <c r="E27">
+        <v>78</v>
+      </c>
+      <c r="D27">
+        <v>5</v>
+      </c>
+      <c r="E27" t="s">
+        <v>207</v>
+      </c>
+      <c r="F27">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C28" t="s">
-        <v>83</v>
-      </c>
-      <c r="D28" t="s">
-        <v>221</v>
-      </c>
-      <c r="E28">
+        <v>78</v>
+      </c>
+      <c r="D28">
+        <v>3</v>
+      </c>
+      <c r="E28" t="s">
+        <v>208</v>
+      </c>
+      <c r="F28">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C29" t="s">
-        <v>83</v>
-      </c>
-      <c r="D29" t="s">
-        <v>222</v>
-      </c>
-      <c r="E29">
+        <v>78</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29" t="s">
+        <v>209</v>
+      </c>
+      <c r="F29">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="C30" t="s">
-        <v>83</v>
-      </c>
-      <c r="D30" t="s">
-        <v>223</v>
-      </c>
-      <c r="E30">
+        <v>78</v>
+      </c>
+      <c r="D30">
+        <v>4</v>
+      </c>
+      <c r="E30" t="s">
+        <v>210</v>
+      </c>
+      <c r="F30">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31" s="17" t="s">
-        <v>89</v>
+      <c r="B31" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="D31" t="s">
-        <v>224</v>
-      </c>
-      <c r="E31">
+        <v>78</v>
+      </c>
+      <c r="D31">
+        <v>4</v>
+      </c>
+      <c r="E31" t="s">
+        <v>211</v>
+      </c>
+      <c r="F31">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="C32" t="s">
-        <v>185</v>
-      </c>
-      <c r="D32" t="s">
-        <v>203</v>
-      </c>
-      <c r="E32">
+        <v>172</v>
+      </c>
+      <c r="D32">
+        <v>5</v>
+      </c>
+      <c r="E32" t="s">
+        <v>190</v>
+      </c>
+      <c r="F32">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>289</v>
+        <v>276</v>
       </c>
       <c r="C33" t="s">
-        <v>185</v>
-      </c>
-      <c r="D33" t="s">
-        <v>204</v>
-      </c>
-      <c r="E33">
+        <v>172</v>
+      </c>
+      <c r="D33">
+        <v>5</v>
+      </c>
+      <c r="E33" t="s">
+        <v>191</v>
+      </c>
+      <c r="F33">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="C34" t="s">
-        <v>185</v>
-      </c>
-      <c r="D34" t="s">
-        <v>208</v>
-      </c>
-      <c r="E34">
+        <v>172</v>
+      </c>
+      <c r="D34">
+        <v>3</v>
+      </c>
+      <c r="E34" t="s">
+        <v>195</v>
+      </c>
+      <c r="F34">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="C35" t="s">
-        <v>185</v>
-      </c>
-      <c r="D35" t="s">
-        <v>209</v>
-      </c>
-      <c r="E35">
+        <v>172</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35" t="s">
+        <v>196</v>
+      </c>
+      <c r="F35">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C43" s="28"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C44" s="28"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C45" s="28"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C46" s="28"/>
-    </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C49" s="29"/>
-    </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C50" s="29"/>
-    </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C51" s="29"/>
-    </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C52" s="29"/>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C43" s="25"/>
+      <c r="D43" s="25"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C44" s="25"/>
+      <c r="D44" s="25"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C45" s="25"/>
+      <c r="D45" s="25"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C46" s="25"/>
+      <c r="D46" s="25"/>
+    </row>
+    <row r="49" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C49" s="26"/>
+      <c r="D49" s="26"/>
+    </row>
+    <row r="50" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C50" s="26"/>
+      <c r="D50" s="26"/>
+    </row>
+    <row r="51" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C51" s="26"/>
+      <c r="D51" s="26"/>
+    </row>
+    <row r="52" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C52" s="26"/>
+      <c r="D52" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4215,401 +4275,295 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D06B9647-6B4F-7F4B-A3D0-2E740D777678}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:C35"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14.1640625" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="5" max="5" width="31.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1</v>
       </c>
       <c r="B10">
         <v>9</v>
       </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>1</v>
       </c>
       <c r="B11">
         <v>10</v>
       </c>
-      <c r="C11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1</v>
       </c>
       <c r="B12">
         <v>11</v>
       </c>
-      <c r="C12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1</v>
       </c>
       <c r="B13">
         <v>12</v>
       </c>
-      <c r="C13">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1</v>
       </c>
       <c r="B14">
         <v>13</v>
       </c>
-      <c r="C14">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1</v>
       </c>
       <c r="B15">
         <v>14</v>
       </c>
-      <c r="C15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1</v>
       </c>
       <c r="B16">
         <v>15</v>
       </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>1</v>
       </c>
       <c r="B17">
         <v>16</v>
       </c>
-      <c r="C17">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>1</v>
       </c>
       <c r="B18">
         <v>17</v>
       </c>
-      <c r="C18">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1</v>
       </c>
       <c r="B19">
         <v>18</v>
       </c>
-      <c r="C19">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1</v>
       </c>
       <c r="B20">
         <v>19</v>
       </c>
-      <c r="C20">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1</v>
       </c>
       <c r="B21">
         <v>20</v>
       </c>
-      <c r="C21">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>1</v>
       </c>
       <c r="B22">
         <v>21</v>
       </c>
-      <c r="C22">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>1</v>
       </c>
       <c r="B23">
         <v>22</v>
       </c>
-      <c r="C23">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>1</v>
       </c>
       <c r="B24">
         <v>23</v>
       </c>
-      <c r="C24">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>1</v>
       </c>
       <c r="B25">
         <v>24</v>
       </c>
-      <c r="C25">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>1</v>
       </c>
       <c r="B26">
         <v>25</v>
       </c>
-      <c r="C26">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>1</v>
       </c>
       <c r="B27">
         <v>26</v>
       </c>
-      <c r="C27">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>1</v>
       </c>
       <c r="B28">
         <v>27</v>
       </c>
-      <c r="C28">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>1</v>
       </c>
       <c r="B29">
         <v>28</v>
       </c>
-      <c r="C29">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>1</v>
       </c>
       <c r="B30">
         <v>29</v>
       </c>
-      <c r="C30">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>1</v>
       </c>
       <c r="B31">
         <v>30</v>
       </c>
-      <c r="C31">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>1</v>
       </c>
       <c r="B32">
         <v>31</v>
       </c>
-      <c r="C32">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>1</v>
       </c>
       <c r="B33">
         <v>32</v>
       </c>
-      <c r="C33">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>1</v>
       </c>
       <c r="B34">
         <v>33</v>
       </c>
-      <c r="C34">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>1</v>
       </c>
       <c r="B35">
         <v>34</v>
-      </c>
-      <c r="C35">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -4624,7 +4578,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD535EB7-4467-3B49-8145-570794BF3025}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:B112"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.1640625" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -4632,10 +4586,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" t="s">
         <v>104</v>
-      </c>
-      <c r="B1" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -5170,7 +5124,7 @@
       <c r="A68">
         <v>10</v>
       </c>
-      <c r="B68" s="22">
+      <c r="B68" s="20">
         <v>1</v>
       </c>
     </row>
@@ -5178,7 +5132,7 @@
       <c r="A69">
         <v>10</v>
       </c>
-      <c r="B69" s="22">
+      <c r="B69" s="20">
         <v>13</v>
       </c>
     </row>
@@ -5186,7 +5140,7 @@
       <c r="A70">
         <v>11</v>
       </c>
-      <c r="B70" s="23">
+      <c r="B70" s="21">
         <v>3</v>
       </c>
     </row>
@@ -5537,7 +5491,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC4C2EFF-02C6-074A-8EA6-4DCC29873E0E}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="15.1640625" customWidth="1"/>
@@ -5547,19 +5501,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B1" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C1" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="D1" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="E1" t="s">
-        <v>179</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -5567,16 +5521,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="D2" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="E2" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -5587,7 +5541,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>120</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -5595,16 +5549,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="C4" t="s">
-        <v>257</v>
+        <v>244</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>178</v>
+        <v>285</v>
       </c>
       <c r="E4" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -5612,16 +5566,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="C5" t="s">
-        <v>256</v>
+        <v>243</v>
       </c>
       <c r="D5" t="s">
-        <v>134</v>
+        <v>284</v>
       </c>
       <c r="E5" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -5629,16 +5583,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="C6" t="s">
-        <v>258</v>
+        <v>245</v>
       </c>
       <c r="D6" t="s">
-        <v>133</v>
+        <v>283</v>
       </c>
       <c r="E6" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -5646,10 +5600,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="D7" t="s">
-        <v>121</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -5657,10 +5611,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="D8" t="s">
-        <v>122</v>
+        <v>287</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -5668,10 +5622,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D9" t="s">
-        <v>123</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -5687,7 +5638,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1DB3B3E-1A0A-CB44-9815-AAA172704B4B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -5701,28 +5652,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="B1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F1" t="s">
         <v>95</v>
       </c>
-      <c r="D1" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1" t="s">
         <v>98</v>
-      </c>
-      <c r="F1" t="s">
-        <v>100</v>
-      </c>
-      <c r="G1" t="s">
-        <v>101</v>
-      </c>
-      <c r="H1" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -5796,7 +5747,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -5811,7 +5762,7 @@
         <v>43190</v>
       </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -5845,7 +5796,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D7" t="s">
         <v>13</v>
@@ -5871,7 +5822,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
@@ -5886,7 +5837,7 @@
         <v>44334</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -5897,7 +5848,7 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D9" t="s">
         <v>8</v>
@@ -5912,7 +5863,7 @@
         <v>45723</v>
       </c>
       <c r="H9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -6027,7 +5978,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="D14" t="s">
         <v>19</v>
@@ -6080,7 +6031,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9F3A7A3-BDA4-9549-81B7-DA9DFB9E098A}">
   <dimension ref="A1:B24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -6088,10 +6039,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="B1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -6111,7 +6062,7 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="24">
+      <c r="A4" s="22">
         <v>3</v>
       </c>
       <c r="B4">
@@ -6207,7 +6158,7 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="25">
+      <c r="A16" s="23">
         <v>8</v>
       </c>
       <c r="B16">
@@ -6271,7 +6222,7 @@
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="25">
+      <c r="A24" s="23">
         <v>14</v>
       </c>
       <c r="B24">
@@ -6289,7 +6240,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{588B1FF2-90F4-704C-B2EA-477ABF81083D}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" customWidth="1"/>
@@ -6300,22 +6251,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="B1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C1" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="D1" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="E1" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="F1" t="s">
-        <v>264</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -6326,16 +6277,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="D2" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="E2" s="4">
         <v>38156</v>
       </c>
       <c r="F2" t="s">
-        <v>265</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -6349,13 +6300,13 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="E3" s="4">
         <v>41422</v>
       </c>
       <c r="F3" t="s">
-        <v>266</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -6366,16 +6317,16 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="D4" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="E4" s="4">
         <v>42447</v>
       </c>
       <c r="F4" t="s">
-        <v>267</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -6386,16 +6337,16 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="D5" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="E5" s="4">
         <v>42668</v>
       </c>
       <c r="F5" t="s">
-        <v>268</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -6406,16 +6357,16 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="D6" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="E6" s="4">
         <v>43199</v>
       </c>
       <c r="F6" t="s">
-        <v>269</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -6426,16 +6377,16 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>161</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>158</v>
+        <v>149</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>146</v>
       </c>
       <c r="E7" s="4">
         <v>43705</v>
       </c>
       <c r="F7" t="s">
-        <v>270</v>
+        <v>257</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -6446,16 +6397,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D8" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="E8" s="4">
         <v>44256</v>
       </c>
       <c r="F8" t="s">
-        <v>271</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -6466,16 +6417,16 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="D9" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="E9" s="4">
         <v>44301</v>
       </c>
       <c r="F9" t="s">
-        <v>272</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -6486,16 +6437,16 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="D10" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="E10" s="4">
         <v>44375</v>
       </c>
       <c r="F10" t="s">
-        <v>273</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -6506,16 +6457,16 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="D11" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
       <c r="E11" s="4">
         <v>44440</v>
       </c>
       <c r="F11" t="s">
-        <v>274</v>
+        <v>261</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -6526,16 +6477,16 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="D12" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
       <c r="E12" s="4">
         <v>45149</v>
       </c>
       <c r="F12" t="s">
-        <v>275</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -6546,16 +6497,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D13" t="s">
-        <v>253</v>
+        <v>240</v>
       </c>
       <c r="E13" s="4">
         <v>45273</v>
       </c>
       <c r="F13" t="s">
-        <v>276</v>
+        <v>263</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -6566,16 +6517,16 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="D14" t="s">
-        <v>253</v>
+        <v>240</v>
       </c>
       <c r="E14" s="4">
         <v>45441</v>
       </c>
       <c r="F14" t="s">
-        <v>277</v>
+        <v>264</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -6586,16 +6537,16 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="D15" t="s">
-        <v>253</v>
+        <v>240</v>
       </c>
       <c r="E15" s="4">
         <v>45492</v>
       </c>
       <c r="F15" t="s">
-        <v>278</v>
+        <v>265</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -6606,16 +6557,16 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="D16" t="s">
-        <v>253</v>
+        <v>240</v>
       </c>
       <c r="E16" s="4">
         <v>45741</v>
       </c>
       <c r="F16" t="s">
-        <v>279</v>
+        <v>266</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -6626,16 +6577,16 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="D17" t="s">
-        <v>253</v>
+        <v>240</v>
       </c>
       <c r="E17" s="4">
         <v>45805</v>
       </c>
       <c r="F17" t="s">
-        <v>280</v>
+        <v>267</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -6646,16 +6597,16 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="D18" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
       <c r="E18" s="4">
         <v>45805</v>
       </c>
       <c r="F18" t="s">
-        <v>281</v>
+        <v>268</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -6666,16 +6617,16 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="D19" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
       <c r="E19" s="4">
         <v>45867</v>
       </c>
       <c r="F19" t="s">
-        <v>282</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -6686,16 +6637,16 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
       <c r="D20" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
       <c r="E20" s="4">
         <v>46108</v>
       </c>
       <c r="F20" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -6718,7 +6669,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AADB0D70-4A30-354E-B1F7-417C7FE3B3BE}">
   <dimension ref="A1:B72"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -6730,10 +6681,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="B1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -7316,11 +7267,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C85F627-DDBE-1742-9905-942D5D2BA886}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:H15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.83203125" customWidth="1"/>
     <col min="4" max="4" width="98.33203125" customWidth="1"/>
     <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.5" bestFit="1" customWidth="1"/>
@@ -7330,28 +7281,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" t="s">
         <v>95</v>
       </c>
-      <c r="D1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G1" t="s">
+        <v>137</v>
+      </c>
+      <c r="H1" t="s">
         <v>100</v>
-      </c>
-      <c r="F1" t="s">
-        <v>101</v>
-      </c>
-      <c r="G1" t="s">
-        <v>149</v>
-      </c>
-      <c r="H1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -7362,10 +7313,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>259</v>
+        <v>246</v>
       </c>
       <c r="D2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E2" s="4">
         <v>42892</v>
@@ -7374,7 +7325,7 @@
         <v>42999</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -7385,10 +7336,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="D3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E3" s="4">
         <v>43915</v>
@@ -7397,7 +7348,7 @@
         <v>44277</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -7408,10 +7359,10 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E4" s="4">
         <v>44331</v>
@@ -7420,10 +7371,10 @@
         <v>45723</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -7434,19 +7385,22 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>296</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
       </c>
       <c r="E5" s="4">
-        <v>45744</v>
-      </c>
-      <c r="G5" t="s">
-        <v>151</v>
-      </c>
-      <c r="H5" t="s">
-        <v>42</v>
+        <v>46028</v>
+      </c>
+      <c r="F5" s="4">
+        <v>46106</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -7457,16 +7411,17 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>64</v>
+        <v>294</v>
       </c>
       <c r="D6" t="s">
-        <v>43</v>
+        <v>289</v>
       </c>
       <c r="E6" s="4">
-        <v>45756</v>
-      </c>
+        <v>46105</v>
+      </c>
+      <c r="F6" s="4"/>
       <c r="G6" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -7477,16 +7432,22 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>65</v>
+        <v>295</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E7" s="4">
         <v>45842</v>
       </c>
-      <c r="G7" t="s">
-        <v>151</v>
+      <c r="F7" s="4">
+        <v>46112</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -7497,19 +7458,19 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>261</v>
+        <v>248</v>
       </c>
       <c r="D8" t="s">
-        <v>251</v>
+        <v>238</v>
       </c>
       <c r="E8" s="4">
         <v>45565</v>
       </c>
       <c r="G8" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="H8" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -7520,19 +7481,19 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="D9" t="s">
-        <v>250</v>
+        <v>237</v>
       </c>
       <c r="E9" s="4">
         <v>45616</v>
       </c>
       <c r="G9" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="H9" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -7543,19 +7504,19 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>263</v>
+        <v>250</v>
       </c>
       <c r="D10" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="E10" s="4">
         <v>45565</v>
       </c>
       <c r="G10" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -7566,19 +7527,19 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="D11" t="s">
-        <v>248</v>
+        <v>235</v>
       </c>
       <c r="E11" s="4">
         <v>45876</v>
       </c>
       <c r="G11" t="s">
-        <v>150</v>
-      </c>
-      <c r="H11" t="s">
-        <v>148</v>
+        <v>138</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -7589,14 +7550,14 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E12" s="4"/>
       <c r="G12" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -7607,16 +7568,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="D13" t="s">
-        <v>249</v>
+        <v>236</v>
       </c>
       <c r="E13" s="4">
         <v>45871</v>
       </c>
       <c r="G13" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -7627,14 +7588,14 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="D14" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E14" s="4"/>
       <c r="G14" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -7645,17 +7606,20 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>295</v>
+        <v>282</v>
       </c>
       <c r="D15" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
       <c r="E15" s="4">
         <v>45901</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" t="s">
-        <v>150</v>
+        <v>138</v>
+      </c>
+      <c r="H15" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -7666,10 +7630,13 @@
     <hyperlink ref="H8" r:id="rId3" xr:uid="{9024645F-B90B-6C49-A5AD-FBDB984D2A47}"/>
     <hyperlink ref="H9" r:id="rId4" xr:uid="{6A990671-87B8-7543-89E2-11F397485368}"/>
     <hyperlink ref="H10" r:id="rId5" xr:uid="{C273DA0B-17C9-0F49-AAE4-F1DFD24E4CA4}"/>
+    <hyperlink ref="H7" r:id="rId6" xr:uid="{38A82EE0-E664-4B49-9718-B5EF47828CDB}"/>
+    <hyperlink ref="H11" r:id="rId7" xr:uid="{160F5AC7-78D1-E347-BC0D-6E1E9E6301BF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7677,7 +7644,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{651096C1-5898-C549-BD57-20844C051C27}">
   <dimension ref="A1:B23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19" bestFit="1" customWidth="1"/>
@@ -7685,10 +7652,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B1" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -7878,486 +7845,568 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCC0C039-730B-9449-8AEE-126A0687A846}">
   <sheetPr codeName="Sheet11"/>
-  <dimension ref="A1:E38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F38"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="25.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" customWidth="1"/>
+    <col min="5" max="5" width="62" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B1" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C1" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D1" t="s">
         <v>103</v>
       </c>
       <c r="E1" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+      <c r="F1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11">
         <v>1</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D2" t="s">
-        <v>225</v>
-      </c>
-      <c r="E2">
+        <v>113</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>168</v>
+      </c>
+      <c r="D2">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>212</v>
+      </c>
+      <c r="F2">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="13">
         <v>2</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D3" t="s">
-        <v>230</v>
-      </c>
-      <c r="E3">
+        <v>43</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D3">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>217</v>
+      </c>
+      <c r="F3">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="11">
         <v>3</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D4" t="s">
-        <v>226</v>
-      </c>
-      <c r="E4">
+        <v>44</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D4">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>213</v>
+      </c>
+      <c r="F4">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="13">
         <v>4</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D5" t="s">
-        <v>227</v>
-      </c>
-      <c r="E5">
+        <v>52</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D5">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F5">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="11">
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" t="s">
-        <v>231</v>
-      </c>
-      <c r="E6">
+        <v>45</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6" t="s">
+        <v>218</v>
+      </c>
+      <c r="F6">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="13">
         <v>6</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" t="s">
-        <v>232</v>
-      </c>
-      <c r="E7">
+        <v>46</v>
+      </c>
+      <c r="C7" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>219</v>
+      </c>
+      <c r="F7">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="11">
         <v>7</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" t="s">
-        <v>228</v>
-      </c>
-      <c r="E8">
+        <v>47</v>
+      </c>
+      <c r="C8" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8">
+        <v>9</v>
+      </c>
+      <c r="E8" t="s">
+        <v>215</v>
+      </c>
+      <c r="F8">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="13">
         <v>8</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D9" t="s">
-        <v>229</v>
-      </c>
-      <c r="E9">
+        <v>68</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D9">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>216</v>
+      </c>
+      <c r="F9">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="11">
         <v>9</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" t="s">
-        <v>233</v>
-      </c>
-      <c r="E10">
+        <v>56</v>
+      </c>
+      <c r="D10">
+        <v>8</v>
+      </c>
+      <c r="E10" t="s">
+        <v>220</v>
+      </c>
+      <c r="F10">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="13">
         <v>10</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D11" t="s">
-        <v>234</v>
-      </c>
-      <c r="E11">
+        <v>49</v>
+      </c>
+      <c r="C11" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D11">
+        <v>9</v>
+      </c>
+      <c r="E11" t="s">
+        <v>221</v>
+      </c>
+      <c r="F11">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="18">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="16">
         <v>11</v>
       </c>
-      <c r="B12" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D12" t="s">
-        <v>235</v>
-      </c>
-      <c r="E12">
+      <c r="B12" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D12">
+        <v>6</v>
+      </c>
+      <c r="E12" t="s">
+        <v>222</v>
+      </c>
+      <c r="F12">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="19">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="17">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D13" t="s">
-        <v>236</v>
-      </c>
-      <c r="E13">
+        <v>50</v>
+      </c>
+      <c r="C13" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13" t="s">
+        <v>223</v>
+      </c>
+      <c r="F13">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="18">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="16">
         <v>13</v>
       </c>
-      <c r="B14" s="21" t="s">
-        <v>188</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D14" t="s">
-        <v>237</v>
-      </c>
-      <c r="E14">
+      <c r="B14" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D14">
+        <v>7</v>
+      </c>
+      <c r="E14" t="s">
+        <v>224</v>
+      </c>
+      <c r="F14">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="19">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="17">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>183</v>
-      </c>
-      <c r="C15" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="D15" t="s">
-        <v>238</v>
-      </c>
-      <c r="E15">
+        <v>170</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15">
+        <v>6</v>
+      </c>
+      <c r="E15" t="s">
+        <v>225</v>
+      </c>
+      <c r="F15">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="18">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="16">
         <v>15</v>
       </c>
-      <c r="B16" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C16" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" t="s">
-        <v>255</v>
-      </c>
-      <c r="E16">
+      <c r="B16" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16">
+        <v>10</v>
+      </c>
+      <c r="E16" t="s">
+        <v>242</v>
+      </c>
+      <c r="F16">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="13">
         <v>16</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="D17" t="s">
-        <v>239</v>
-      </c>
-      <c r="E17">
+        <v>70</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="D17">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
+        <v>226</v>
+      </c>
+      <c r="F17">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="13">
         <v>17</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="D18" t="s">
-        <v>240</v>
-      </c>
-      <c r="E18">
+        <v>109</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="D18">
+        <v>9</v>
+      </c>
+      <c r="E18" t="s">
+        <v>227</v>
+      </c>
+      <c r="F18">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="13">
         <v>18</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="D19" t="s">
-        <v>241</v>
-      </c>
-      <c r="E19">
+        <v>110</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="D19">
+        <v>8</v>
+      </c>
+      <c r="E19" t="s">
+        <v>228</v>
+      </c>
+      <c r="F19">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="13">
         <v>19</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="D20" t="s">
-        <v>242</v>
-      </c>
-      <c r="E20">
+        <v>112</v>
+      </c>
+      <c r="C20" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="D20">
+        <v>8</v>
+      </c>
+      <c r="E20" t="s">
+        <v>229</v>
+      </c>
+      <c r="F20">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="13">
         <v>20</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="D21" t="s">
-        <v>243</v>
-      </c>
-      <c r="E21">
+        <v>111</v>
+      </c>
+      <c r="C21" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="D21">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>230</v>
+      </c>
+      <c r="F21">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="20">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="18">
         <v>21</v>
       </c>
-      <c r="B22" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="D22" t="s">
-        <v>244</v>
-      </c>
-      <c r="E22">
+      <c r="B22" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="D22">
+        <v>6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>231</v>
+      </c>
+      <c r="F22">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="20">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="18">
         <v>22</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="C23" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="D23" t="s">
-        <v>245</v>
-      </c>
-      <c r="E23">
+      <c r="B23" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="C23" s="27" t="s">
+        <v>168</v>
+      </c>
+      <c r="D23">
+        <v>8</v>
+      </c>
+      <c r="E23" t="s">
+        <v>232</v>
+      </c>
+      <c r="F23">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="20">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="18">
         <v>23</v>
       </c>
-      <c r="B24" s="21" t="s">
-        <v>190</v>
-      </c>
-      <c r="C24" s="31" t="s">
-        <v>181</v>
-      </c>
-      <c r="D24" t="s">
-        <v>246</v>
-      </c>
-      <c r="E24">
+      <c r="B24" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="C24" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="D24">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
+        <v>233</v>
+      </c>
+      <c r="F24">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="20">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="18">
         <v>24</v>
       </c>
-      <c r="B25" s="21" t="s">
-        <v>287</v>
-      </c>
-      <c r="C25" s="31" t="s">
-        <v>181</v>
-      </c>
-      <c r="D25" t="s">
-        <v>288</v>
-      </c>
-      <c r="E25">
+      <c r="B25" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="C25" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="D25">
+        <v>6</v>
+      </c>
+      <c r="E25" t="s">
+        <v>275</v>
+      </c>
+      <c r="F25">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C31" s="28"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C32" s="28"/>
-    </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C33" s="28"/>
-    </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C36" s="29"/>
-    </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C37" s="29"/>
-    </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C38" s="29"/>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+    </row>
+    <row r="33" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+    </row>
+    <row r="36" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C36" s="26"/>
+      <c r="D36" s="26"/>
+    </row>
+    <row r="37" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C37" s="26"/>
+      <c r="D37" s="26"/>
+    </row>
+    <row r="38" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C38" s="26"/>
+      <c r="D38" s="26"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update binary files for master database; executed pipeline.
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2525185F-5315-E947-981A-B32C83E1325B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71AE39DF-FEEB-624E-9FFB-51AB1EEBA5F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28500" windowHeight="28200" firstSheet="1" activeTab="6" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" firstSheet="1" activeTab="1" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -423,9 +423,6 @@
     <t>Funding Consultant</t>
   </si>
   <si>
-    <t>I thrive at the intersection of science, innovation and data. My path taught me to adapt quickly, communicate effectively and create impact in diverse contexts. Along the way, I learned to shape projects strategically and make complex information accessible through clear visualization and storytelling.</t>
-  </si>
-  <si>
     <t>Schleswig-Holstein</t>
   </si>
   <si>
@@ -543,9 +540,6 @@
     <t>#Innovation #FundingStrategy #ProjectManagement</t>
   </si>
   <si>
-    <t>#DataScience #Insights #Visualization</t>
-  </si>
-  <si>
     <t>#Science #Microalgae #Sustainability</t>
   </si>
   <si>
@@ -900,24 +894,12 @@
     <t>ZIM-Network for    Bioeconomy</t>
   </si>
   <si>
-    <t>Processed and analyzed large biological datasets. Designed reproducible data workflows and scientific models using Python (statistical analysis, multivariate techniques). Published results in peer-reviewed journals.</t>
-  </si>
-  <si>
-    <t>Advised clients on innovation strategies and technology-driven projects, including AI and data-related applications (from idea framing to successful funding acquisition). Collaborated with cross-functional stake-holders across industry &amp; research.</t>
-  </si>
-  <si>
-    <t>Explored a complex phototropic system which is used for sustainable bioremediation (water cleaning) through academic biotechnological research. Sharpened skills in problem-solving, experimental design and data analysis. Published results in peer-reviewed journals.</t>
-  </si>
-  <si>
     <t>As a hobby, I create games focusing on model creation (Blender) and engine coding (Unity).</t>
   </si>
   <si>
     <t>As a lecturer, I gave students insights into the field of general molecular biology.</t>
   </si>
   <si>
-    <t>After graduation, I specialist into the field of biology. Explored the beauty and detailness of animals, plants and microorganisms.</t>
-  </si>
-  <si>
     <t>Physiological responses of floc-forming microalgae-bacteria consortia to environmental perturbations</t>
   </si>
   <si>
@@ -940,6 +922,24 @@
   </si>
   <si>
     <t>Paper in Algal    Research</t>
+  </si>
+  <si>
+    <t>Following my graduation, I specialized in the field of biology, where I explored the intricate beauty and detailed mechanisms of animals, plants, and microorganisms. This focus allowed me to delve deep into the natural world while building a robust foundation in life sciences.</t>
+  </si>
+  <si>
+    <t>Following my graduation, I specialized in the field of biology, where I explored the beauty and detailed mechanisms of animals, plants and microorganisms.</t>
+  </si>
+  <si>
+    <t>My research journey led me to investigate a complex phototropic system designed for sustainable bioremediation, specifically for water cleaning. Through academic biotechnological research, I sharpened my skills in problem-solving, experimental design and data analysis. Finally, I published my findings in peer-reviewed journals to contribute to the broader scientific community.</t>
+  </si>
+  <si>
+    <t>I advise clients on innovation strategies and technology-driven projects, including AI and data-related applications. My role spans the entire lifecycle from collaboratively framing initial ideas into successfully funded projects. In this capacity, I collaborate closely with cross-functional stakeholders across both industry and research sectors to help bridge the gap between theoretical potential and practical implementation.</t>
+  </si>
+  <si>
+    <t>I processed and analyzed large-scale biological datasets to uncover meaningful patterns. I designed reproducible data workflows and developed scientific models using Python, employing statistical analysis and multivariate techniques. Finally, I published my findings in peer-reviewed journals to contribute to the broader scientific community.</t>
+  </si>
+  <si>
+    <t>#DataAnalysis #Python #DataVisualization</t>
   </si>
 </sst>
 </file>
@@ -1311,6 +1311,12 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1357,12 +1363,6 @@
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1387,7 +1387,7 @@
     <tableColumn id="6" xr3:uid="{08E97EF2-2A58-9142-81F6-5F4A1B6CAF2C}" name="city"/>
     <tableColumn id="5" xr3:uid="{831CB986-42F5-9D46-860A-8100DBA32197}" name="province"/>
     <tableColumn id="4" xr3:uid="{7564C2FC-BB92-7742-A00C-C96E922B28EF}" name="country"/>
-    <tableColumn id="9" xr3:uid="{C61E8E18-A34B-F64D-911A-EB79E1C91129}" name="birth_date" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{C61E8E18-A34B-F64D-911A-EB79E1C91129}" name="birth_date" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1495,8 +1495,8 @@
     <tableColumn id="3" xr3:uid="{519CB3FD-482A-2B44-9C5A-9E797E3F98E4}" name="title"/>
     <tableColumn id="4" xr3:uid="{0DBFEBFC-D18A-6F4E-87F2-C8D4D16C7E2D}" name="organization"/>
     <tableColumn id="9" xr3:uid="{3E657E01-C34B-0B41-8B45-85D9AE50305B}" name="location"/>
-    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="8"/>
     <tableColumn id="8" xr3:uid="{4B60B559-FFE2-0449-BD87-E423F2579CE2}" name="description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1507,7 +1507,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}" name="Table14" displayName="Table14" ref="A1:B24" totalsRowShown="0">
   <autoFilter ref="A1:B24" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{647E29E8-3B30-6747-952B-856B15C586DD}" name="domain_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1548,8 +1548,8 @@
     <tableColumn id="6" xr3:uid="{D37906CD-C2EB-8A40-AA51-891ADDD2F0F3}" name="person_id"/>
     <tableColumn id="8" xr3:uid="{912FC1CE-8929-A840-BCE1-17117B008FD3}" name="title"/>
     <tableColumn id="11" xr3:uid="{8675359A-ECB9-7944-B6E4-F8EFBA93E841}" name="description"/>
-    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="10"/>
-    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="9"/>
+    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="5"/>
     <tableColumn id="1" xr3:uid="{D859FDAD-79F9-EC41-ACD6-64B4107CA00A}" name="status"/>
     <tableColumn id="12" xr3:uid="{267EBF1D-F600-6746-8520-55E6EE075513}" name="link"/>
   </tableColumns>
@@ -1934,13 +1934,13 @@
         <v>92</v>
       </c>
       <c r="E1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F1" t="s">
+        <v>126</v>
+      </c>
+      <c r="G1" t="s">
         <v>127</v>
-      </c>
-      <c r="G1" t="s">
-        <v>128</v>
       </c>
       <c r="H1" t="s">
         <v>94</v>
@@ -1960,13 +1960,13 @@
         <v>88</v>
       </c>
       <c r="E2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F2" t="s">
+        <v>124</v>
+      </c>
+      <c r="G2" t="s">
         <v>125</v>
-      </c>
-      <c r="G2" t="s">
-        <v>126</v>
       </c>
       <c r="H2" s="4">
         <v>34220</v>
@@ -3511,7 +3511,7 @@
         <v>98</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
@@ -3526,13 +3526,13 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D2">
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F2">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3547,13 +3547,13 @@
         <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D3">
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F3">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3565,16 +3565,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D4">
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F4">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3586,16 +3586,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C5" t="s">
         <v>171</v>
       </c>
-      <c r="C5" t="s">
-        <v>173</v>
-      </c>
       <c r="D5">
         <v>3</v>
       </c>
       <c r="E5" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F5">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3610,13 +3610,13 @@
         <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D6">
         <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F6">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3631,13 +3631,13 @@
         <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F7">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3652,13 +3652,13 @@
         <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F8">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3673,13 +3673,13 @@
         <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F9">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3694,13 +3694,13 @@
         <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F10">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3715,13 +3715,13 @@
         <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
       <c r="E11" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="F11">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3736,13 +3736,13 @@
         <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D12">
         <v>2</v>
       </c>
       <c r="E12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F12">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3754,16 +3754,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C13" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D13">
         <v>5</v>
       </c>
       <c r="E13" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F13">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3778,13 +3778,13 @@
         <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D14">
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="F14">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3805,7 +3805,7 @@
         <v>3</v>
       </c>
       <c r="E15" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F15">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3826,7 +3826,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F16">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3847,7 +3847,7 @@
         <v>3</v>
       </c>
       <c r="E17" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F17">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3862,13 +3862,13 @@
         <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D18">
         <v>3</v>
       </c>
       <c r="E18" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="F18">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3880,16 +3880,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C19" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D19">
         <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="F19">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3904,13 +3904,13 @@
         <v>53</v>
       </c>
       <c r="C20" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D20">
         <v>3</v>
       </c>
       <c r="E20" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F20">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3925,13 +3925,13 @@
         <v>54</v>
       </c>
       <c r="C21" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D21">
         <v>3</v>
       </c>
       <c r="E21" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F21">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3952,7 +3952,7 @@
         <v>5</v>
       </c>
       <c r="E22" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F22">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3973,7 +3973,7 @@
         <v>4</v>
       </c>
       <c r="E23" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F23">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3994,7 +3994,7 @@
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F24">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4015,7 +4015,7 @@
         <v>3</v>
       </c>
       <c r="E25" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F25">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4027,7 +4027,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C26" t="s">
         <v>78</v>
@@ -4036,7 +4036,7 @@
         <v>5</v>
       </c>
       <c r="E26" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F26">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4048,7 +4048,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C27" t="s">
         <v>78</v>
@@ -4057,7 +4057,7 @@
         <v>5</v>
       </c>
       <c r="E27" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F27">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4078,7 +4078,7 @@
         <v>3</v>
       </c>
       <c r="E28" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F28">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4099,7 +4099,7 @@
         <v>3</v>
       </c>
       <c r="E29" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F29">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4120,7 +4120,7 @@
         <v>4</v>
       </c>
       <c r="E30" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F30">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4141,7 +4141,7 @@
         <v>4</v>
       </c>
       <c r="E31" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F31">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4153,16 +4153,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C32" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D32">
         <v>5</v>
       </c>
       <c r="E32" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F32">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4174,16 +4174,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C33" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D33">
         <v>5</v>
       </c>
       <c r="E33" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F33">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4195,16 +4195,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C34" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D34">
         <v>3</v>
       </c>
       <c r="E34" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="F34">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4216,16 +4216,16 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C35" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="D35">
         <v>4</v>
       </c>
       <c r="E35" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F35">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -5513,7 +5513,7 @@
         <v>98</v>
       </c>
       <c r="E1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -5524,13 +5524,13 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E2" t="s">
         <v>161</v>
-      </c>
-      <c r="D2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -5541,7 +5541,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -5552,13 +5552,13 @@
         <v>118</v>
       </c>
       <c r="C4" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="E4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -5569,13 +5569,13 @@
         <v>123</v>
       </c>
       <c r="C5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D5" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="E5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -5586,13 +5586,13 @@
         <v>120</v>
       </c>
       <c r="C6" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D6" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="E6" t="s">
-        <v>164</v>
+        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -5603,7 +5603,7 @@
         <v>119</v>
       </c>
       <c r="D7" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -5614,7 +5614,7 @@
         <v>121</v>
       </c>
       <c r="D8" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -5628,6 +5628,7 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -6251,7 +6252,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" t="s">
         <v>89</v>
@@ -6260,13 +6261,13 @@
         <v>116</v>
       </c>
       <c r="D1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F1" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -6277,16 +6278,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E2" s="4">
         <v>38156</v>
       </c>
       <c r="F2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -6300,13 +6301,13 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E3" s="4">
         <v>41422</v>
       </c>
       <c r="F3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -6317,16 +6318,16 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E4" s="4">
         <v>42447</v>
       </c>
       <c r="F4" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -6337,16 +6338,16 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E5" s="4">
         <v>42668</v>
       </c>
       <c r="F5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -6357,16 +6358,16 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E6" s="4">
         <v>43199</v>
       </c>
       <c r="F6" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -6377,16 +6378,16 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E7" s="4">
         <v>43705</v>
       </c>
       <c r="F7" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -6397,16 +6398,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E8" s="4">
         <v>44256</v>
       </c>
       <c r="F8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -6417,16 +6418,16 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E9" s="4">
         <v>44301</v>
       </c>
       <c r="F9" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -6437,16 +6438,16 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E10" s="4">
         <v>44375</v>
       </c>
       <c r="F10" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -6457,16 +6458,16 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D11" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E11" s="4">
         <v>44440</v>
       </c>
       <c r="F11" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -6477,16 +6478,16 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D12" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E12" s="4">
         <v>45149</v>
       </c>
       <c r="F12" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -6497,16 +6498,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D13" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E13" s="4">
         <v>45273</v>
       </c>
       <c r="F13" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -6517,16 +6518,16 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D14" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E14" s="4">
         <v>45441</v>
       </c>
       <c r="F14" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -6537,16 +6538,16 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D15" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E15" s="4">
         <v>45492</v>
       </c>
       <c r="F15" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -6557,16 +6558,16 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D16" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E16" s="4">
         <v>45741</v>
       </c>
       <c r="F16" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -6577,16 +6578,16 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D17" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E17" s="4">
         <v>45805</v>
       </c>
       <c r="F17" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -6597,16 +6598,16 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D18" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E18" s="4">
         <v>45805</v>
       </c>
       <c r="F18" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -6617,16 +6618,16 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D19" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="E19" s="4">
         <v>45867</v>
       </c>
       <c r="F19" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -6637,16 +6638,16 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E20" s="4">
         <v>46108</v>
       </c>
       <c r="F20" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -6681,7 +6682,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1" t="s">
         <v>114</v>
@@ -7299,7 +7300,7 @@
         <v>96</v>
       </c>
       <c r="G1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H1" t="s">
         <v>100</v>
@@ -7313,7 +7314,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D2" t="s">
         <v>60</v>
@@ -7325,7 +7326,7 @@
         <v>42999</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -7336,7 +7337,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D3" t="s">
         <v>59</v>
@@ -7348,7 +7349,7 @@
         <v>44277</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -7371,7 +7372,7 @@
         <v>45723</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>63</v>
@@ -7385,7 +7386,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -7397,10 +7398,10 @@
         <v>46106</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -7411,17 +7412,17 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="D6" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="E6" s="4">
         <v>46105</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -7432,7 +7433,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="D7" t="s">
         <v>42</v>
@@ -7444,10 +7445,10 @@
         <v>46112</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -7458,16 +7459,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E8" s="4">
         <v>45565</v>
       </c>
       <c r="G8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H8" t="s">
         <v>64</v>
@@ -7481,16 +7482,16 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D9" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E9" s="4">
         <v>45616</v>
       </c>
       <c r="G9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H9" t="s">
         <v>65</v>
@@ -7504,19 +7505,19 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D10" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E10" s="4">
         <v>45565</v>
       </c>
       <c r="G10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -7527,19 +7528,19 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D11" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E11" s="4">
         <v>45876</v>
       </c>
       <c r="G11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -7550,14 +7551,14 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D12" t="s">
         <v>61</v>
       </c>
       <c r="E12" s="4"/>
       <c r="G12" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -7568,16 +7569,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D13" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E13" s="4">
         <v>45871</v>
       </c>
       <c r="G13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -7588,14 +7589,14 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D14" t="s">
         <v>62</v>
       </c>
       <c r="E14" s="4"/>
       <c r="G14" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -7606,20 +7607,20 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="D15" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="E15" s="4">
         <v>45901</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H15" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>
@@ -7877,7 +7878,7 @@
         <v>98</v>
       </c>
       <c r="F1" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -7888,13 +7889,13 @@
         <v>113</v>
       </c>
       <c r="C2" s="29" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D2">
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F2">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -7909,13 +7910,13 @@
         <v>43</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D3">
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F3">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -7930,13 +7931,13 @@
         <v>44</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D4">
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F4">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -7951,13 +7952,13 @@
         <v>52</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D5">
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F5">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -7978,7 +7979,7 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F6">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -7999,7 +8000,7 @@
         <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="F7">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8020,7 +8021,7 @@
         <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F8">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8035,13 +8036,13 @@
         <v>68</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D9">
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F9">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8062,7 +8063,7 @@
         <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F10">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8077,13 +8078,13 @@
         <v>49</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D11">
         <v>9</v>
       </c>
       <c r="E11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F11">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8098,13 +8099,13 @@
         <v>66</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D12">
         <v>6</v>
       </c>
       <c r="E12" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F12">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8119,13 +8120,13 @@
         <v>50</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D13">
         <v>8</v>
       </c>
       <c r="E13" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F13">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8137,16 +8138,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D14">
         <v>7</v>
       </c>
       <c r="E14" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F14">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8158,7 +8159,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C15" s="28" t="s">
         <v>56</v>
@@ -8167,7 +8168,7 @@
         <v>6</v>
       </c>
       <c r="E15" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="F15">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8188,7 +8189,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F16">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8203,13 +8204,13 @@
         <v>70</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D17">
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F17">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8224,13 +8225,13 @@
         <v>109</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D18">
         <v>9</v>
       </c>
       <c r="E18" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F18">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8245,13 +8246,13 @@
         <v>110</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D19">
         <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F19">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8266,13 +8267,13 @@
         <v>112</v>
       </c>
       <c r="C20" s="28" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D20">
         <v>8</v>
       </c>
       <c r="E20" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F20">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8287,13 +8288,13 @@
         <v>111</v>
       </c>
       <c r="C21" s="28" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D21">
         <v>7</v>
       </c>
       <c r="E21" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F21">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8308,13 +8309,13 @@
         <v>71</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D22">
         <v>6</v>
       </c>
       <c r="E22" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F22">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8326,16 +8327,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D23">
         <v>8</v>
       </c>
       <c r="E23" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="F23">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8347,16 +8348,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D24">
         <v>7</v>
       </c>
       <c r="E24" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F24">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8368,16 +8369,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C25" s="30" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D25">
         <v>6</v>
       </c>
       <c r="E25" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F25">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>

</xml_diff>

<commit_message>
Update database domain descriptions; executed pipeline
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71AE39DF-FEEB-624E-9FFB-51AB1EEBA5F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB9709B-5292-0E4D-A42D-3A54A4ABBA4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" firstSheet="1" activeTab="1" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
@@ -924,9 +924,6 @@
     <t>Paper in Algal    Research</t>
   </si>
   <si>
-    <t>Following my graduation, I specialized in the field of biology, where I explored the intricate beauty and detailed mechanisms of animals, plants, and microorganisms. This focus allowed me to delve deep into the natural world while building a robust foundation in life sciences.</t>
-  </si>
-  <si>
     <t>Following my graduation, I specialized in the field of biology, where I explored the beauty and detailed mechanisms of animals, plants and microorganisms.</t>
   </si>
   <si>
@@ -940,6 +937,9 @@
   </si>
   <si>
     <t>#DataAnalysis #Python #DataVisualization</t>
+  </si>
+  <si>
+    <t>I thrive at the intersection of science, innovation, and data. My path taught me to adapt quickly, communicate effectively and create serious impact across diverse contexts. Along my way, I have learned to shape projects strategically and transform complex information into accessible insights through clear visualization and compelling storytelling.</t>
   </si>
 </sst>
 </file>
@@ -5527,7 +5527,7 @@
         <v>160</v>
       </c>
       <c r="D2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E2" t="s">
         <v>161</v>
@@ -5541,7 +5541,7 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -5555,7 +5555,7 @@
         <v>242</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E4" t="s">
         <v>163</v>
@@ -5572,7 +5572,7 @@
         <v>241</v>
       </c>
       <c r="D5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E5" t="s">
         <v>162</v>
@@ -5589,10 +5589,10 @@
         <v>243</v>
       </c>
       <c r="D6" t="s">
+        <v>294</v>
+      </c>
+      <c r="E6" t="s">
         <v>295</v>
-      </c>
-      <c r="E6" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update database bug fixed; executed pipeline.
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB9709B-5292-0E4D-A42D-3A54A4ABBA4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E44108F-255F-B445-8961-F89069380C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" firstSheet="1" activeTab="1" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
@@ -939,7 +939,7 @@
     <t>#DataAnalysis #Python #DataVisualization</t>
   </si>
   <si>
-    <t>I thrive at the intersection of science, innovation, and data. My path taught me to adapt quickly, communicate effectively and create serious impact across diverse contexts. Along my way, I have learned to shape projects strategically and transform complex information into accessible insights through clear visualization and compelling storytelling.</t>
+    <t>I thrive at the intersection of science, innovation and data. My path taught me to adapt quickly, communicate effectively and create serious impact across diverse contexts. Along my way, I have learned to shape projects strategically and transform complex information into accessible insights through clear visualization and compelling storytelling.</t>
   </si>
 </sst>
 </file>
@@ -950,7 +950,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -993,6 +993,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1156,7 +1161,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1188,6 +1193,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5527,7 +5533,7 @@
         <v>160</v>
       </c>
       <c r="D2" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="E2" t="s">
         <v>161</v>
@@ -5540,8 +5546,8 @@
       <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
-        <v>296</v>
+      <c r="D3" s="31" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Master database adaption in domain description; executed pipeline
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E44108F-255F-B445-8961-F89069380C04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1101C2-F163-B040-9109-D56611BCCF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" firstSheet="1" activeTab="1" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
@@ -927,19 +927,19 @@
     <t>Following my graduation, I specialized in the field of biology, where I explored the beauty and detailed mechanisms of animals, plants and microorganisms.</t>
   </si>
   <si>
-    <t>My research journey led me to investigate a complex phototropic system designed for sustainable bioremediation, specifically for water cleaning. Through academic biotechnological research, I sharpened my skills in problem-solving, experimental design and data analysis. Finally, I published my findings in peer-reviewed journals to contribute to the broader scientific community.</t>
-  </si>
-  <si>
-    <t>I advise clients on innovation strategies and technology-driven projects, including AI and data-related applications. My role spans the entire lifecycle from collaboratively framing initial ideas into successfully funded projects. In this capacity, I collaborate closely with cross-functional stakeholders across both industry and research sectors to help bridge the gap between theoretical potential and practical implementation.</t>
-  </si>
-  <si>
-    <t>I processed and analyzed large-scale biological datasets to uncover meaningful patterns. I designed reproducible data workflows and developed scientific models using Python, employing statistical analysis and multivariate techniques. Finally, I published my findings in peer-reviewed journals to contribute to the broader scientific community.</t>
-  </si>
-  <si>
     <t>#DataAnalysis #Python #DataVisualization</t>
   </si>
   <si>
     <t>I thrive at the intersection of science, innovation and data. My path taught me to adapt quickly, communicate effectively and create serious impact across diverse contexts. Along my way, I have learned to shape projects strategically and transform complex information into accessible insights through clear visualization and compelling storytelling.</t>
+  </si>
+  <si>
+    <t>My research journey led me to investigate a complex phototropic system designed for sustainable bioremediation, specifically for water cleaning. Through academic biotechnological research, I sharpened my skills in problem-solving, experimental design and data analysis. Finally, I published my findings in peer-reviewed journals.</t>
+  </si>
+  <si>
+    <t>I advise clients on innovation strategies and technology-driven projects, including AI and data-related applications. My role spans the entire lifecycle from collaboratively framing initial ideas into successfully funded projects. In this capacity, I collaborate closely with cross-functional stakeholders across both industry and research sectors.</t>
+  </si>
+  <si>
+    <t>I processed and analyzed large-scale biological datasets (metagenomic sequencing data) to uncover meaningful patterns. I designed reproducible data workflows and developed scientific models using Python, employing statistical analysis and multivariate techniques. Finally, I published my findings in peer-reviewed journals.</t>
   </si>
 </sst>
 </file>
@@ -5533,7 +5533,7 @@
         <v>160</v>
       </c>
       <c r="D2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="E2" t="s">
         <v>161</v>
@@ -5561,7 +5561,7 @@
         <v>242</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E4" t="s">
         <v>163</v>
@@ -5578,7 +5578,7 @@
         <v>241</v>
       </c>
       <c r="D5" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E5" t="s">
         <v>162</v>
@@ -5595,10 +5595,10 @@
         <v>243</v>
       </c>
       <c r="D6" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E6" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update master database (domain activity relation of doctorate); executed pipeline
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1101C2-F163-B040-9109-D56611BCCF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE52C90D-BB30-1E40-BB24-02775B5A88B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" firstSheet="1" activeTab="1" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" firstSheet="1" activeTab="3" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -1510,8 +1510,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}" name="Table14" displayName="Table14" ref="A1:B24" totalsRowShown="0">
-  <autoFilter ref="A1:B24" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}" name="Table14" displayName="Table14" ref="A1:B23" totalsRowShown="0">
+  <autoFilter ref="A1:B23" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{647E29E8-3B30-6747-952B-856B15C586DD}" name="domain_id"/>
@@ -6037,7 +6037,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9F3A7A3-BDA4-9549-81B7-DA9DFB9E098A}">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
@@ -6165,24 +6165,24 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="23">
-        <v>8</v>
+      <c r="A16" s="11">
+        <v>9</v>
       </c>
       <c r="B16">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B17">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B18">
         <v>2</v>
@@ -6190,7 +6190,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="11">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B19">
         <v>2</v>
@@ -6201,38 +6201,30 @@
         <v>12</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B21">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B22">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="11">
+      <c r="A23" s="23">
         <v>14</v>
       </c>
       <c r="B23">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="23">
-        <v>14</v>
-      </c>
-      <c r="B24">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "Master database adaption in domain description; executed pipeline"
This reverts commit df5622b51cccae64a7e17669feb87aa64ad56eeb.
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE52C90D-BB30-1E40-BB24-02775B5A88B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1101C2-F163-B040-9109-D56611BCCF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" firstSheet="1" activeTab="3" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" firstSheet="1" activeTab="1" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -1510,8 +1510,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}" name="Table14" displayName="Table14" ref="A1:B23" totalsRowShown="0">
-  <autoFilter ref="A1:B23" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}" name="Table14" displayName="Table14" ref="A1:B24" totalsRowShown="0">
+  <autoFilter ref="A1:B24" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{647E29E8-3B30-6747-952B-856B15C586DD}" name="domain_id"/>
@@ -6037,7 +6037,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9F3A7A3-BDA4-9549-81B7-DA9DFB9E098A}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
@@ -6165,24 +6165,24 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="11">
-        <v>9</v>
+      <c r="A16" s="23">
+        <v>8</v>
       </c>
       <c r="B16">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B17">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="11">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B18">
         <v>2</v>
@@ -6190,7 +6190,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="11">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B19">
         <v>2</v>
@@ -6201,30 +6201,38 @@
         <v>12</v>
       </c>
       <c r="B20">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="11">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="11">
+        <v>13</v>
+      </c>
+      <c r="B22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="11">
         <v>14</v>
       </c>
-      <c r="B22">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="23">
+      <c r="B23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="23">
         <v>14</v>
       </c>
-      <c r="B23">
+      <c r="B24">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Published Version 2.0 now includes: - Live data connection via Google Sheets - Implemented single offline database export file as alternative - Update README.md
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1101C2-F163-B040-9109-D56611BCCF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E6100D-CEF3-9D40-9CBB-FB5D3D68648B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" firstSheet="1" activeTab="1" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="10" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="297">
   <si>
     <t>Graduation</t>
   </si>
@@ -333,9 +333,6 @@
     <t>location</t>
   </si>
   <si>
-    <t>birth_date</t>
-  </si>
-  <si>
     <t>start_date</t>
   </si>
   <si>
@@ -888,9 +885,6 @@
     <t>Agentic coding, python &amp; C# programming, jupyter notebook</t>
   </si>
   <si>
-    <t>Data Analysis (SQL, BI &amp; Excel)</t>
-  </si>
-  <si>
     <t>ZIM-Network for    Bioeconomy</t>
   </si>
   <si>
@@ -940,6 +934,12 @@
   </si>
   <si>
     <t>I processed and analyzed large-scale biological datasets (metagenomic sequencing data) to uncover meaningful patterns. I designed reproducible data workflows and developed scientific models using Python, employing statistical analysis and multivariate techniques. Finally, I published my findings in peer-reviewed journals.</t>
+  </si>
+  <si>
+    <t>Consultant</t>
+  </si>
+  <si>
+    <t>Data Analysis        (SQL, BI &amp; Excel)</t>
   </si>
 </sst>
 </file>
@@ -1200,7 +1200,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="10">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1366,9 +1366,6 @@
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1383,9 +1380,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9D7F923B-7B23-7B4C-9250-DE534D0C77CD}" name="Table1" displayName="Table1" ref="A1:H2" totalsRowShown="0">
-  <autoFilter ref="A1:H2" xr:uid="{9D7F923B-7B23-7B4C-9250-DE534D0C77CD}"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9D7F923B-7B23-7B4C-9250-DE534D0C77CD}" name="Table1" displayName="Table1" ref="A1:G2" totalsRowShown="0">
+  <autoFilter ref="A1:G2" xr:uid="{9D7F923B-7B23-7B4C-9250-DE534D0C77CD}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{60B9BDE2-8505-464B-922F-D796FBEFDBA8}" name="person_id"/>
     <tableColumn id="8" xr3:uid="{EF244F48-5D7D-1849-A5A5-EFB52CEE84E2}" name="title"/>
     <tableColumn id="2" xr3:uid="{5BEB6B06-7483-FF4F-810F-5649A2FBD651}" name="first_name"/>
@@ -1393,7 +1390,6 @@
     <tableColumn id="6" xr3:uid="{08E97EF2-2A58-9142-81F6-5F4A1B6CAF2C}" name="city"/>
     <tableColumn id="5" xr3:uid="{831CB986-42F5-9D46-860A-8100DBA32197}" name="province"/>
     <tableColumn id="4" xr3:uid="{7564C2FC-BB92-7742-A00C-C96E922B28EF}" name="country"/>
-    <tableColumn id="9" xr3:uid="{C61E8E18-A34B-F64D-911A-EB79E1C91129}" name="birth_date" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1411,8 +1407,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DEA382D8-61D8-844C-A457-95EAB096446A}" name="Table8" displayName="Table8" ref="A1:B156" totalsRowShown="0">
-  <autoFilter ref="A1:B156" xr:uid="{DEA382D8-61D8-844C-A457-95EAB096446A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DEA382D8-61D8-844C-A457-95EAB096446A}" name="Table8" displayName="Table8" ref="A1:B165" totalsRowShown="0">
+  <autoFilter ref="A1:B165" xr:uid="{DEA382D8-61D8-844C-A457-95EAB096446A}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{05D161FC-81FA-D643-8CB1-172DCE26A4E3}" name="portfolio_id"/>
     <tableColumn id="2" xr3:uid="{C5E6A4B1-46AB-3840-B226-F474361FE659}" name="skill_id"/>
@@ -1912,7 +1908,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA051E34-3D1F-4D4A-8D3B-9B3E0598856B}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -1922,11 +1918,10 @@
     <col min="5" max="5" width="13.1640625" customWidth="1"/>
     <col min="6" max="6" width="37" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="37" customWidth="1"/>
-    <col min="8" max="8" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="20.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -1940,19 +1935,16 @@
         <v>92</v>
       </c>
       <c r="E1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G1" t="s">
         <v>126</v>
       </c>
-      <c r="G1" t="s">
-        <v>127</v>
-      </c>
-      <c r="H1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1966,16 +1958,13 @@
         <v>88</v>
       </c>
       <c r="E2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" t="s">
         <v>124</v>
-      </c>
-      <c r="G2" t="s">
-        <v>125</v>
-      </c>
-      <c r="H2" s="4">
-        <v>34220</v>
       </c>
     </row>
   </sheetData>
@@ -2008,7 +1997,7 @@
         <v>89</v>
       </c>
       <c r="B1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
@@ -2221,7 +2210,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C6AC091-0337-EE42-81A2-CB3A7445D977}">
   <sheetPr codeName="Sheet10"/>
-  <dimension ref="A1:B156"/>
+  <dimension ref="A1:B165"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
@@ -2230,10 +2219,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -3474,6 +3463,78 @@
       </c>
       <c r="B156">
         <v>24</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A157">
+        <v>14</v>
+      </c>
+      <c r="B157">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A158">
+        <v>14</v>
+      </c>
+      <c r="B158">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A159">
+        <v>14</v>
+      </c>
+      <c r="B159">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A160">
+        <v>14</v>
+      </c>
+      <c r="B160">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A161">
+        <v>14</v>
+      </c>
+      <c r="B161">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A162">
+        <v>14</v>
+      </c>
+      <c r="B162">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A163">
+        <v>14</v>
+      </c>
+      <c r="B163">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A164">
+        <v>14</v>
+      </c>
+      <c r="B164">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A165">
+        <v>14</v>
+      </c>
+      <c r="B165">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -3502,22 +3563,22 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D1" t="s">
         <v>102</v>
       </c>
-      <c r="D1" t="s">
-        <v>103</v>
-      </c>
       <c r="E1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
@@ -3532,13 +3593,13 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D2">
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F2">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3553,13 +3614,13 @@
         <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D3">
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F3">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3571,16 +3632,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D4">
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F4">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3592,16 +3653,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5">
         <v>3</v>
       </c>
       <c r="E5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F5">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3616,13 +3677,13 @@
         <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D6">
         <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F6">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3637,13 +3698,13 @@
         <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F7">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3658,13 +3719,13 @@
         <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F8">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3679,13 +3740,13 @@
         <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F9">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3700,13 +3761,13 @@
         <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F10">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3721,13 +3782,13 @@
         <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
       <c r="E11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F11">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3742,13 +3803,13 @@
         <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D12">
         <v>2</v>
       </c>
       <c r="E12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F12">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3760,16 +3821,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D13">
         <v>5</v>
       </c>
       <c r="E13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F13">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3784,13 +3845,13 @@
         <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D14">
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F14">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3811,7 +3872,7 @@
         <v>3</v>
       </c>
       <c r="E15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F15">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3832,7 +3893,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F16">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3853,7 +3914,7 @@
         <v>3</v>
       </c>
       <c r="E17" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F17">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3868,13 +3929,13 @@
         <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D18">
         <v>3</v>
       </c>
       <c r="E18" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F18">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3886,16 +3947,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C19" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D19">
         <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F19">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3910,13 +3971,13 @@
         <v>53</v>
       </c>
       <c r="C20" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D20">
         <v>3</v>
       </c>
       <c r="E20" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F20">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3931,13 +3992,13 @@
         <v>54</v>
       </c>
       <c r="C21" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D21">
         <v>3</v>
       </c>
       <c r="E21" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F21">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3958,7 +4019,7 @@
         <v>5</v>
       </c>
       <c r="E22" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F22">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3979,7 +4040,7 @@
         <v>4</v>
       </c>
       <c r="E23" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F23">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4000,7 +4061,7 @@
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F24">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4021,7 +4082,7 @@
         <v>3</v>
       </c>
       <c r="E25" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F25">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4033,7 +4094,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C26" t="s">
         <v>78</v>
@@ -4042,7 +4103,7 @@
         <v>5</v>
       </c>
       <c r="E26" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F26">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4054,7 +4115,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C27" t="s">
         <v>78</v>
@@ -4063,7 +4124,7 @@
         <v>5</v>
       </c>
       <c r="E27" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F27">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4084,7 +4145,7 @@
         <v>3</v>
       </c>
       <c r="E28" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F28">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4105,7 +4166,7 @@
         <v>3</v>
       </c>
       <c r="E29" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F29">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4117,7 +4178,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C30" t="s">
         <v>78</v>
@@ -4126,7 +4187,7 @@
         <v>4</v>
       </c>
       <c r="E30" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F30">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4147,7 +4208,7 @@
         <v>4</v>
       </c>
       <c r="E31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F31">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4159,16 +4220,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C32" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D32">
         <v>5</v>
       </c>
       <c r="E32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F32">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4180,16 +4241,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C33" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D33">
         <v>5</v>
       </c>
       <c r="E33" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F33">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4201,16 +4262,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C34" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D34">
         <v>3</v>
       </c>
       <c r="E34" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F34">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4222,16 +4283,16 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C35" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D35">
         <v>4</v>
       </c>
       <c r="E35" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F35">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4297,7 +4358,7 @@
         <v>89</v>
       </c>
       <c r="B1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -4592,10 +4653,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -5507,19 +5568,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -5530,13 +5591,13 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D2" t="s">
+        <v>291</v>
+      </c>
+      <c r="E2" t="s">
         <v>160</v>
-      </c>
-      <c r="D2" t="s">
-        <v>293</v>
-      </c>
-      <c r="E2" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -5547,7 +5608,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -5555,16 +5616,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="E4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -5572,16 +5633,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>123</v>
+        <v>295</v>
       </c>
       <c r="C5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -5589,16 +5650,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D6" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="E6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -5606,10 +5667,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -5617,10 +5678,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D8" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -5659,7 +5720,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1" t="s">
         <v>89</v>
@@ -5668,19 +5729,19 @@
         <v>90</v>
       </c>
       <c r="D1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E1" t="s">
         <v>93</v>
       </c>
       <c r="F1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G1" t="s">
         <v>95</v>
       </c>
-      <c r="G1" t="s">
-        <v>96</v>
-      </c>
       <c r="H1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -5754,7 +5815,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -5803,7 +5864,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D7" t="s">
         <v>13</v>
@@ -5829,7 +5890,7 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
@@ -5855,7 +5916,7 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D9" t="s">
         <v>8</v>
@@ -5985,7 +6046,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D14" t="s">
         <v>19</v>
@@ -6046,10 +6107,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -6258,22 +6319,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1" t="s">
         <v>89</v>
       </c>
       <c r="C1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -6284,16 +6345,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E2" s="4">
         <v>38156</v>
       </c>
       <c r="F2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -6307,13 +6368,13 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E3" s="4">
         <v>41422</v>
       </c>
       <c r="F3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -6324,16 +6385,16 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E4" s="4">
         <v>42447</v>
       </c>
       <c r="F4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -6344,16 +6405,16 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E5" s="4">
         <v>42668</v>
       </c>
       <c r="F5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -6364,16 +6425,16 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E6" s="4">
         <v>43199</v>
       </c>
       <c r="F6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -6384,16 +6445,16 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E7" s="4">
         <v>43705</v>
       </c>
       <c r="F7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -6404,16 +6465,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E8" s="4">
         <v>44256</v>
       </c>
       <c r="F8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -6424,16 +6485,16 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E9" s="4">
         <v>44301</v>
       </c>
       <c r="F9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -6444,16 +6505,16 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E10" s="4">
         <v>44375</v>
       </c>
       <c r="F10" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -6464,16 +6525,16 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D11" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E11" s="4">
         <v>44440</v>
       </c>
       <c r="F11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -6484,16 +6545,16 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D12" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E12" s="4">
         <v>45149</v>
       </c>
       <c r="F12" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -6504,16 +6565,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E13" s="4">
         <v>45273</v>
       </c>
       <c r="F13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -6524,16 +6585,16 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E14" s="4">
         <v>45441</v>
       </c>
       <c r="F14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -6544,16 +6605,16 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D15" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E15" s="4">
         <v>45492</v>
       </c>
       <c r="F15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -6564,16 +6625,16 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D16" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E16" s="4">
         <v>45741</v>
       </c>
       <c r="F16" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -6584,16 +6645,16 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D17" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E17" s="4">
         <v>45805</v>
       </c>
       <c r="F17" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -6604,16 +6665,16 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D18" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E18" s="4">
         <v>45805</v>
       </c>
       <c r="F18" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -6624,16 +6685,16 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>279</v>
+        <v>296</v>
       </c>
       <c r="D19" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E19" s="4">
         <v>45867</v>
       </c>
       <c r="F19" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -6644,16 +6705,16 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" t="s">
         <v>268</v>
-      </c>
-      <c r="D20" t="s">
-        <v>269</v>
       </c>
       <c r="E20" s="4">
         <v>46108</v>
       </c>
       <c r="F20" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -6688,10 +6749,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -7288,7 +7349,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B1" t="s">
         <v>89</v>
@@ -7297,19 +7358,19 @@
         <v>90</v>
       </c>
       <c r="D1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F1" t="s">
         <v>95</v>
       </c>
-      <c r="F1" t="s">
-        <v>96</v>
-      </c>
       <c r="G1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -7320,7 +7381,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D2" t="s">
         <v>60</v>
@@ -7332,7 +7393,7 @@
         <v>42999</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -7343,7 +7404,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D3" t="s">
         <v>59</v>
@@ -7355,7 +7416,7 @@
         <v>44277</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -7378,7 +7439,7 @@
         <v>45723</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>63</v>
@@ -7392,7 +7453,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -7404,10 +7465,10 @@
         <v>46106</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -7418,17 +7479,17 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E6" s="4">
         <v>46105</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -7439,7 +7500,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D7" t="s">
         <v>42</v>
@@ -7451,10 +7512,10 @@
         <v>46112</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -7465,16 +7526,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E8" s="4">
         <v>45565</v>
       </c>
       <c r="G8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H8" t="s">
         <v>64</v>
@@ -7488,16 +7549,16 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E9" s="4">
         <v>45616</v>
       </c>
       <c r="G9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H9" t="s">
         <v>65</v>
@@ -7511,19 +7572,19 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E10" s="4">
         <v>45565</v>
       </c>
       <c r="G10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -7534,19 +7595,19 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D11" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E11" s="4">
         <v>45876</v>
       </c>
       <c r="G11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -7557,14 +7618,14 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D12" t="s">
         <v>61</v>
       </c>
       <c r="E12" s="4"/>
       <c r="G12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -7575,16 +7636,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D13" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E13" s="4">
         <v>45871</v>
       </c>
       <c r="G13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -7595,14 +7656,14 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D14" t="s">
         <v>62</v>
       </c>
       <c r="E14" s="4"/>
       <c r="G14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -7613,20 +7674,20 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D15" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E15" s="4">
         <v>45901</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H15" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -7659,10 +7720,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -7869,22 +7930,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" t="s">
         <v>101</v>
       </c>
-      <c r="B1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>102</v>
       </c>
-      <c r="D1" t="s">
-        <v>103</v>
-      </c>
       <c r="E1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -7892,16 +7953,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C2" s="29" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D2">
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F2">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -7916,13 +7977,13 @@
         <v>43</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D3">
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F3">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -7937,17 +7998,17 @@
         <v>44</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D4">
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F4">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -7958,17 +8019,17 @@
         <v>52</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D5">
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F5">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -7985,11 +8046,11 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F6">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -8006,7 +8067,7 @@
         <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F7">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8027,11 +8088,11 @@
         <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F8">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -8042,17 +8103,17 @@
         <v>68</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D9">
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F9">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -8069,7 +8130,7 @@
         <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F10">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8084,13 +8145,13 @@
         <v>49</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D11">
         <v>9</v>
       </c>
       <c r="E11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F11">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8105,17 +8166,17 @@
         <v>66</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D12">
         <v>6</v>
       </c>
       <c r="E12" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F12">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -8126,13 +8187,13 @@
         <v>50</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D13">
         <v>8</v>
       </c>
       <c r="E13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F13">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8144,20 +8205,20 @@
         <v>13</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D14">
         <v>7</v>
       </c>
       <c r="E14" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F14">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -8165,7 +8226,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C15" s="28" t="s">
         <v>56</v>
@@ -8174,11 +8235,11 @@
         <v>6</v>
       </c>
       <c r="E15" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F15">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -8195,11 +8256,11 @@
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F16">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -8210,13 +8271,13 @@
         <v>70</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D17">
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F17">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8228,16 +8289,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D18">
         <v>9</v>
       </c>
       <c r="E18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F18">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8249,16 +8310,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D19">
         <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F19">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8270,16 +8331,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C20" s="28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D20">
         <v>8</v>
       </c>
       <c r="E20" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F20">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8291,16 +8352,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C21" s="28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D21">
         <v>7</v>
       </c>
       <c r="E21" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F21">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8315,13 +8376,13 @@
         <v>71</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D22">
         <v>6</v>
       </c>
       <c r="E22" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F22">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8333,16 +8394,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D23">
         <v>8</v>
       </c>
       <c r="E23" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F23">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8354,16 +8415,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D24">
         <v>7</v>
       </c>
       <c r="E24" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F24">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8375,16 +8436,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C25" s="30" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D25">
         <v>6</v>
       </c>
       <c r="E25" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F25">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>

</xml_diff>

<commit_message>
Fixed date format bug. Executed pipeline.
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0E6100D-CEF3-9D40-9CBB-FB5D3D68648B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A8A99F4-CC6D-F443-8FD0-158F213F2DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="10" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="6" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -402,9 +402,6 @@
     <t>Bioreactor Systems</t>
   </si>
   <si>
-    <t>Biologist</t>
-  </si>
-  <si>
     <t>Game Developer</t>
   </si>
   <si>
@@ -940,6 +937,9 @@
   </si>
   <si>
     <t>Data Analysis        (SQL, BI &amp; Excel)</t>
+  </si>
+  <si>
+    <t>Researcher</t>
   </si>
 </sst>
 </file>
@@ -1935,13 +1935,13 @@
         <v>92</v>
       </c>
       <c r="E1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G1" t="s">
         <v>125</v>
-      </c>
-      <c r="G1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -1958,13 +1958,13 @@
         <v>88</v>
       </c>
       <c r="E2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" t="s">
         <v>123</v>
-      </c>
-      <c r="G2" t="s">
-        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3578,7 +3578,7 @@
         <v>97</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
@@ -3593,13 +3593,13 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D2">
         <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F2">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3614,13 +3614,13 @@
         <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D3">
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F3">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3632,16 +3632,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D4">
         <v>3</v>
       </c>
       <c r="E4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F4">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3653,16 +3653,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D5">
         <v>3</v>
       </c>
       <c r="E5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F5">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3677,13 +3677,13 @@
         <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D6">
         <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F6">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3698,13 +3698,13 @@
         <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F7">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3719,13 +3719,13 @@
         <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F8">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3740,13 +3740,13 @@
         <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F9">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3761,13 +3761,13 @@
         <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F10">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3782,13 +3782,13 @@
         <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
       <c r="E11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F11">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3803,13 +3803,13 @@
         <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D12">
         <v>2</v>
       </c>
       <c r="E12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F12">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3821,16 +3821,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D13">
         <v>5</v>
       </c>
       <c r="E13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F13">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3845,13 +3845,13 @@
         <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D14">
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F14">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3872,7 +3872,7 @@
         <v>3</v>
       </c>
       <c r="E15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F15">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3893,7 +3893,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F16">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3914,7 +3914,7 @@
         <v>3</v>
       </c>
       <c r="E17" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F17">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3929,13 +3929,13 @@
         <v>40</v>
       </c>
       <c r="C18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D18">
         <v>3</v>
       </c>
       <c r="E18" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F18">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3947,16 +3947,16 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D19">
         <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F19">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3971,13 +3971,13 @@
         <v>53</v>
       </c>
       <c r="C20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D20">
         <v>3</v>
       </c>
       <c r="E20" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F20">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3992,13 +3992,13 @@
         <v>54</v>
       </c>
       <c r="C21" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D21">
         <v>3</v>
       </c>
       <c r="E21" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F21">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4019,7 +4019,7 @@
         <v>5</v>
       </c>
       <c r="E22" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F22">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4040,7 +4040,7 @@
         <v>4</v>
       </c>
       <c r="E23" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F23">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4061,7 +4061,7 @@
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F24">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4082,7 +4082,7 @@
         <v>3</v>
       </c>
       <c r="E25" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F25">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4094,7 +4094,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C26" t="s">
         <v>78</v>
@@ -4103,7 +4103,7 @@
         <v>5</v>
       </c>
       <c r="E26" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F26">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4115,7 +4115,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C27" t="s">
         <v>78</v>
@@ -4124,7 +4124,7 @@
         <v>5</v>
       </c>
       <c r="E27" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F27">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4145,7 +4145,7 @@
         <v>3</v>
       </c>
       <c r="E28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F28">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4166,7 +4166,7 @@
         <v>3</v>
       </c>
       <c r="E29" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F29">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4187,7 +4187,7 @@
         <v>4</v>
       </c>
       <c r="E30" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F30">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4208,7 +4208,7 @@
         <v>4</v>
       </c>
       <c r="E31" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F31">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4220,16 +4220,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C32" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D32">
         <v>5</v>
       </c>
       <c r="E32" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F32">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4241,16 +4241,16 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C33" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D33">
         <v>5</v>
       </c>
       <c r="E33" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F33">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4262,16 +4262,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C34" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D34">
         <v>3</v>
       </c>
       <c r="E34" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F34">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4283,16 +4283,16 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C35" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D35">
         <v>4</v>
       </c>
       <c r="E35" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F35">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -5574,13 +5574,13 @@
         <v>115</v>
       </c>
       <c r="C1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D1" t="s">
         <v>97</v>
       </c>
       <c r="E1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -5591,13 +5591,13 @@
         <v>69</v>
       </c>
       <c r="C2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D2" t="s">
+        <v>290</v>
+      </c>
+      <c r="E2" t="s">
         <v>159</v>
-      </c>
-      <c r="D2" t="s">
-        <v>291</v>
-      </c>
-      <c r="E2" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -5608,7 +5608,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -5616,16 +5616,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>117</v>
+        <v>296</v>
       </c>
       <c r="C4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -5633,16 +5633,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -5650,16 +5650,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -5667,10 +5667,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -5678,10 +5678,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -6046,7 +6046,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D14" t="s">
         <v>19</v>
@@ -6319,7 +6319,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1" t="s">
         <v>89</v>
@@ -6328,13 +6328,13 @@
         <v>115</v>
       </c>
       <c r="D1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -6345,16 +6345,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E2" s="4">
         <v>38156</v>
       </c>
       <c r="F2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -6368,13 +6368,13 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E3" s="4">
         <v>41422</v>
       </c>
       <c r="F3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -6385,16 +6385,16 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E4" s="4">
         <v>42447</v>
       </c>
       <c r="F4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -6405,16 +6405,16 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E5" s="4">
         <v>42668</v>
       </c>
       <c r="F5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -6425,16 +6425,16 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E6" s="4">
         <v>43199</v>
       </c>
       <c r="F6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -6445,16 +6445,16 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E7" s="4">
         <v>43705</v>
       </c>
       <c r="F7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -6465,16 +6465,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E8" s="4">
         <v>44256</v>
       </c>
       <c r="F8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -6485,16 +6485,16 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D9" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E9" s="4">
         <v>44301</v>
       </c>
       <c r="F9" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -6505,16 +6505,16 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E10" s="4">
         <v>44375</v>
       </c>
       <c r="F10" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -6525,16 +6525,16 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D11" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E11" s="4">
         <v>44440</v>
       </c>
       <c r="F11" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -6545,16 +6545,16 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D12" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E12" s="4">
         <v>45149</v>
       </c>
       <c r="F12" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -6565,16 +6565,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E13" s="4">
         <v>45273</v>
       </c>
       <c r="F13" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -6585,16 +6585,16 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D14" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E14" s="4">
         <v>45441</v>
       </c>
       <c r="F14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -6605,16 +6605,16 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D15" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E15" s="4">
         <v>45492</v>
       </c>
       <c r="F15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -6625,16 +6625,16 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D16" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E16" s="4">
         <v>45741</v>
       </c>
       <c r="F16" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -6645,16 +6645,16 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D17" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E17" s="4">
         <v>45805</v>
       </c>
       <c r="F17" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -6665,16 +6665,16 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D18" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E18" s="4">
         <v>45805</v>
       </c>
       <c r="F18" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -6685,16 +6685,16 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D19" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E19" s="4">
         <v>45867</v>
       </c>
       <c r="F19" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -6705,16 +6705,16 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
+        <v>266</v>
+      </c>
+      <c r="D20" t="s">
         <v>267</v>
-      </c>
-      <c r="D20" t="s">
-        <v>268</v>
       </c>
       <c r="E20" s="4">
         <v>46108</v>
       </c>
       <c r="F20" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -6749,7 +6749,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1" t="s">
         <v>113</v>
@@ -7367,7 +7367,7 @@
         <v>95</v>
       </c>
       <c r="G1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H1" t="s">
         <v>99</v>
@@ -7381,7 +7381,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D2" t="s">
         <v>60</v>
@@ -7393,7 +7393,7 @@
         <v>42999</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -7404,7 +7404,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D3" t="s">
         <v>59</v>
@@ -7416,7 +7416,7 @@
         <v>44277</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -7439,7 +7439,7 @@
         <v>45723</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>63</v>
@@ -7453,7 +7453,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -7465,10 +7465,10 @@
         <v>46106</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -7479,17 +7479,17 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E6" s="4">
         <v>46105</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -7500,7 +7500,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D7" t="s">
         <v>42</v>
@@ -7512,10 +7512,10 @@
         <v>46112</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -7526,16 +7526,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E8" s="4">
         <v>45565</v>
       </c>
       <c r="G8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H8" t="s">
         <v>64</v>
@@ -7549,16 +7549,16 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E9" s="4">
         <v>45616</v>
       </c>
       <c r="G9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H9" t="s">
         <v>65</v>
@@ -7572,19 +7572,19 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D10" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E10" s="4">
         <v>45565</v>
       </c>
       <c r="G10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -7595,19 +7595,19 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D11" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E11" s="4">
         <v>45876</v>
       </c>
       <c r="G11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -7618,14 +7618,14 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D12" t="s">
         <v>61</v>
       </c>
       <c r="E12" s="4"/>
       <c r="G12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -7636,16 +7636,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E13" s="4">
         <v>45871</v>
       </c>
       <c r="G13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -7656,14 +7656,14 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D14" t="s">
         <v>62</v>
       </c>
       <c r="E14" s="4"/>
       <c r="G14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -7674,20 +7674,20 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D15" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E15" s="4">
         <v>45901</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H15" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>
@@ -7945,7 +7945,7 @@
         <v>97</v>
       </c>
       <c r="F1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -7956,13 +7956,13 @@
         <v>112</v>
       </c>
       <c r="C2" s="29" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D2">
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F2">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -7977,13 +7977,13 @@
         <v>43</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D3">
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F3">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -7998,13 +7998,13 @@
         <v>44</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D4">
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F4">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8019,13 +8019,13 @@
         <v>52</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D5">
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F5">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8046,7 +8046,7 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F6">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8067,7 +8067,7 @@
         <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F7">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8088,7 +8088,7 @@
         <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F8">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8103,13 +8103,13 @@
         <v>68</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D9">
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F9">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8130,7 +8130,7 @@
         <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F10">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8145,13 +8145,13 @@
         <v>49</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D11">
         <v>9</v>
       </c>
       <c r="E11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F11">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8166,13 +8166,13 @@
         <v>66</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D12">
         <v>6</v>
       </c>
       <c r="E12" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F12">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8187,13 +8187,13 @@
         <v>50</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D13">
         <v>8</v>
       </c>
       <c r="E13" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F13">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8205,16 +8205,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D14">
         <v>7</v>
       </c>
       <c r="E14" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F14">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8226,7 +8226,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C15" s="28" t="s">
         <v>56</v>
@@ -8235,7 +8235,7 @@
         <v>6</v>
       </c>
       <c r="E15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F15">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8256,7 +8256,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F16">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8271,13 +8271,13 @@
         <v>70</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D17">
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F17">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8292,13 +8292,13 @@
         <v>108</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D18">
         <v>9</v>
       </c>
       <c r="E18" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F18">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8313,13 +8313,13 @@
         <v>109</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D19">
         <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F19">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8334,13 +8334,13 @@
         <v>111</v>
       </c>
       <c r="C20" s="28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D20">
         <v>8</v>
       </c>
       <c r="E20" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F20">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8355,13 +8355,13 @@
         <v>110</v>
       </c>
       <c r="C21" s="28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D21">
         <v>7</v>
       </c>
       <c r="E21" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F21">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8376,13 +8376,13 @@
         <v>71</v>
       </c>
       <c r="C22" s="28" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D22">
         <v>6</v>
       </c>
       <c r="E22" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F22">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8394,16 +8394,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D23">
         <v>8</v>
       </c>
       <c r="E23" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F23">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8415,16 +8415,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C24" s="28" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D24">
         <v>7</v>
       </c>
       <c r="E24" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F24">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8436,16 +8436,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C25" s="30" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D25">
         <v>6</v>
       </c>
       <c r="E25" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F25">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>

</xml_diff>

<commit_message>
Added new certificate (QGIS) to database Executed pipeline Minor readme changes
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A8A99F4-CC6D-F443-8FD0-158F213F2DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B3D408-1EA1-B940-ACE5-1B40CD013F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="6" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="4" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="299">
   <si>
     <t>Graduation</t>
   </si>
@@ -940,6 +940,12 @@
   </si>
   <si>
     <t>Researcher</t>
+  </si>
+  <si>
+    <t>QGIS: Beginner to Advanced</t>
+  </si>
+  <si>
+    <t>2026-06-02_Udemy_QGIS.jpg</t>
   </si>
 </sst>
 </file>
@@ -1317,12 +1323,6 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1359,6 +1359,12 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
@@ -1497,8 +1503,8 @@
     <tableColumn id="3" xr3:uid="{519CB3FD-482A-2B44-9C5A-9E797E3F98E4}" name="title"/>
     <tableColumn id="4" xr3:uid="{0DBFEBFC-D18A-6F4E-87F2-C8D4D16C7E2D}" name="organization"/>
     <tableColumn id="9" xr3:uid="{3E657E01-C34B-0B41-8B45-85D9AE50305B}" name="location"/>
-    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="6"/>
     <tableColumn id="8" xr3:uid="{4B60B559-FFE2-0449-BD87-E423F2579CE2}" name="description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1509,7 +1515,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}" name="Table14" displayName="Table14" ref="A1:B24" totalsRowShown="0">
   <autoFilter ref="A1:B24" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{647E29E8-3B30-6747-952B-856B15C586DD}" name="domain_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1550,8 +1556,8 @@
     <tableColumn id="6" xr3:uid="{D37906CD-C2EB-8A40-AA51-891ADDD2F0F3}" name="person_id"/>
     <tableColumn id="8" xr3:uid="{912FC1CE-8929-A840-BCE1-17117B008FD3}" name="title"/>
     <tableColumn id="11" xr3:uid="{8675359A-ECB9-7944-B6E4-F8EFBA93E841}" name="description"/>
-    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="6"/>
-    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="9"/>
+    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="8"/>
     <tableColumn id="1" xr3:uid="{D859FDAD-79F9-EC41-ACD6-64B4107CA00A}" name="status"/>
     <tableColumn id="12" xr3:uid="{267EBF1D-F600-6746-8520-55E6EE075513}" name="link"/>
   </tableColumns>
@@ -6307,7 +6313,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{588B1FF2-90F4-704C-B2EA-477ABF81083D}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -6718,13 +6724,33 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E21" s="4"/>
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>297</v>
+      </c>
+      <c r="D21" t="s">
+        <v>235</v>
+      </c>
+      <c r="E21" s="4">
+        <v>46175</v>
+      </c>
+      <c r="F21" t="s">
+        <v>298</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E22" s="4"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E24" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added domain link of new certificate Executed pipeline
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5B3D408-1EA1-B940-ACE5-1B40CD013F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E64DC1-F8FB-B24D-B0FB-0642CFF65B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="4" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="5" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -1323,6 +1323,12 @@
       </border>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1359,12 +1365,6 @@
         <vertical/>
         <horizontal/>
       </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
@@ -1503,8 +1503,8 @@
     <tableColumn id="3" xr3:uid="{519CB3FD-482A-2B44-9C5A-9E797E3F98E4}" name="title"/>
     <tableColumn id="4" xr3:uid="{0DBFEBFC-D18A-6F4E-87F2-C8D4D16C7E2D}" name="organization"/>
     <tableColumn id="9" xr3:uid="{3E657E01-C34B-0B41-8B45-85D9AE50305B}" name="location"/>
-    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="8"/>
     <tableColumn id="8" xr3:uid="{4B60B559-FFE2-0449-BD87-E423F2579CE2}" name="description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1515,7 +1515,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}" name="Table14" displayName="Table14" ref="A1:B24" totalsRowShown="0">
   <autoFilter ref="A1:B24" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{647E29E8-3B30-6747-952B-856B15C586DD}" name="domain_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1538,8 +1538,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A1F68B62-CEBE-6546-949E-F98D282A2879}" name="Table2" displayName="Table2" ref="A1:B72" totalsRowShown="0">
-  <autoFilter ref="A1:B72" xr:uid="{A1F68B62-CEBE-6546-949E-F98D282A2879}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A1F68B62-CEBE-6546-949E-F98D282A2879}" name="Table2" displayName="Table2" ref="A1:B74" totalsRowShown="0">
+  <autoFilter ref="A1:B74" xr:uid="{A1F68B62-CEBE-6546-949E-F98D282A2879}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{A84E7ECA-C8B9-4943-A15E-09A98C9BCFBE}" name="certificate_id"/>
     <tableColumn id="2" xr3:uid="{E364EA32-FECF-2944-9614-C481D07B1732}" name="domain_id"/>
@@ -1556,8 +1556,8 @@
     <tableColumn id="6" xr3:uid="{D37906CD-C2EB-8A40-AA51-891ADDD2F0F3}" name="person_id"/>
     <tableColumn id="8" xr3:uid="{912FC1CE-8929-A840-BCE1-17117B008FD3}" name="title"/>
     <tableColumn id="11" xr3:uid="{8675359A-ECB9-7944-B6E4-F8EFBA93E841}" name="description"/>
-    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="8"/>
+    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="5"/>
     <tableColumn id="1" xr3:uid="{D859FDAD-79F9-EC41-ACD6-64B4107CA00A}" name="status"/>
     <tableColumn id="12" xr3:uid="{267EBF1D-F600-6746-8520-55E6EE075513}" name="link"/>
   </tableColumns>
@@ -6762,7 +6762,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AADB0D70-4A30-354E-B1F7-417C7FE3B3BE}">
-  <dimension ref="A1:B72"/>
+  <dimension ref="A1:B74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -7346,6 +7346,22 @@
         <v>19</v>
       </c>
       <c r="B72">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>20</v>
+      </c>
+      <c r="B73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>20</v>
+      </c>
+      <c r="B74">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Minor fixes including - replaced slim with wide buttons - certificate naming formatting - replaced current resume screenshot for portfolio highlight preview - grammar/wording fixes - date formatting in timeline and certificates
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E64DC1-F8FB-B24D-B0FB-0642CFF65B97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6C0E84-25E4-5145-8351-58891A775BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="5" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="11" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -630,9 +630,6 @@
     <t>literature management, citation organization, research documentation</t>
   </si>
   <si>
-    <t>agile task management, project tracking, documentation</t>
-  </si>
-  <si>
     <t>knowledge base creation, meeting documentation, collaboration</t>
   </si>
   <si>
@@ -642,9 +639,6 @@
     <t>imaging, imageJ, fiji</t>
   </si>
   <si>
-    <t>fluorescence &amp; z-stack imaging</t>
-  </si>
-  <si>
     <t>surface morphology analysis</t>
   </si>
   <si>
@@ -870,18 +864,12 @@
     <t>MS PowerPoint</t>
   </si>
   <si>
-    <t>Trello | MS Planner</t>
-  </si>
-  <si>
     <t>MS Excel</t>
   </si>
   <si>
     <t>MS Word</t>
   </si>
   <si>
-    <t>Agentic coding, python &amp; C# programming, jupyter notebook</t>
-  </si>
-  <si>
     <t>ZIM-Network for    Bioeconomy</t>
   </si>
   <si>
@@ -936,9 +924,6 @@
     <t>Consultant</t>
   </si>
   <si>
-    <t>Data Analysis        (SQL, BI &amp; Excel)</t>
-  </si>
-  <si>
     <t>Researcher</t>
   </si>
   <si>
@@ -946,6 +931,21 @@
   </si>
   <si>
     <t>2026-06-02_Udemy_QGIS.jpg</t>
+  </si>
+  <si>
+    <t>Data Analysis           (SQL, BI &amp; Excel)</t>
+  </si>
+  <si>
+    <t>MS Planner</t>
+  </si>
+  <si>
+    <t>agentic coding, python &amp; C# programming, jupyter notebook</t>
+  </si>
+  <si>
+    <t>agile tasks, project tracking, documentation</t>
+  </si>
+  <si>
+    <t>fluorescence imaging, z-stack imaging</t>
   </si>
 </sst>
 </file>
@@ -3584,7 +3584,7 @@
         <v>97</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
@@ -3827,7 +3827,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C13" t="s">
         <v>168</v>
@@ -3857,7 +3857,7 @@
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>276</v>
+        <v>296</v>
       </c>
       <c r="F14">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3953,7 +3953,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>273</v>
+        <v>295</v>
       </c>
       <c r="C19" t="s">
         <v>168</v>
@@ -3962,7 +3962,7 @@
         <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>193</v>
+        <v>297</v>
       </c>
       <c r="F19">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3983,7 +3983,7 @@
         <v>3</v>
       </c>
       <c r="E20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F20">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4004,7 +4004,7 @@
         <v>3</v>
       </c>
       <c r="E21" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F21">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4025,7 +4025,7 @@
         <v>5</v>
       </c>
       <c r="E22" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F22">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4046,7 +4046,7 @@
         <v>4</v>
       </c>
       <c r="E23" t="s">
-        <v>197</v>
+        <v>298</v>
       </c>
       <c r="F23">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4067,7 +4067,7 @@
         <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F24">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4088,7 +4088,7 @@
         <v>3</v>
       </c>
       <c r="E25" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F25">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4100,7 +4100,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C26" t="s">
         <v>78</v>
@@ -4109,7 +4109,7 @@
         <v>5</v>
       </c>
       <c r="E26" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="F26">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4121,7 +4121,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C27" t="s">
         <v>78</v>
@@ -4130,7 +4130,7 @@
         <v>5</v>
       </c>
       <c r="E27" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F27">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4151,7 +4151,7 @@
         <v>3</v>
       </c>
       <c r="E28" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F28">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4172,7 +4172,7 @@
         <v>3</v>
       </c>
       <c r="E29" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F29">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4193,7 +4193,7 @@
         <v>4</v>
       </c>
       <c r="E30" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F30">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4214,7 +4214,7 @@
         <v>4</v>
       </c>
       <c r="E31" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F31">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4226,7 +4226,7 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C32" t="s">
         <v>168</v>
@@ -4247,7 +4247,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C33" t="s">
         <v>168</v>
@@ -5600,7 +5600,7 @@
         <v>158</v>
       </c>
       <c r="D2" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="E2" t="s">
         <v>159</v>
@@ -5614,7 +5614,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -5622,13 +5622,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="C4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="E4" t="s">
         <v>161</v>
@@ -5639,13 +5639,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="C5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="E5" t="s">
         <v>160</v>
@@ -5659,13 +5659,13 @@
         <v>118</v>
       </c>
       <c r="C6" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D6" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="E6" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -5676,7 +5676,7 @@
         <v>117</v>
       </c>
       <c r="D7" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -5687,7 +5687,7 @@
         <v>119</v>
       </c>
       <c r="D8" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -6340,7 +6340,7 @@
         <v>139</v>
       </c>
       <c r="F1" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -6360,7 +6360,7 @@
         <v>38156</v>
       </c>
       <c r="F2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -6380,7 +6380,7 @@
         <v>41422</v>
       </c>
       <c r="F3" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -6400,7 +6400,7 @@
         <v>42447</v>
       </c>
       <c r="F4" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -6420,7 +6420,7 @@
         <v>42668</v>
       </c>
       <c r="F5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -6440,7 +6440,7 @@
         <v>43199</v>
       </c>
       <c r="F6" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -6460,7 +6460,7 @@
         <v>43705</v>
       </c>
       <c r="F7" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -6480,7 +6480,7 @@
         <v>44256</v>
       </c>
       <c r="F8" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -6500,7 +6500,7 @@
         <v>44301</v>
       </c>
       <c r="F9" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -6520,7 +6520,7 @@
         <v>44375</v>
       </c>
       <c r="F10" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -6534,13 +6534,13 @@
         <v>151</v>
       </c>
       <c r="D11" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E11" s="4">
         <v>44440</v>
       </c>
       <c r="F11" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -6554,13 +6554,13 @@
         <v>152</v>
       </c>
       <c r="D12" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E12" s="4">
         <v>45149</v>
       </c>
       <c r="F12" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -6574,13 +6574,13 @@
         <v>153</v>
       </c>
       <c r="D13" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E13" s="4">
         <v>45273</v>
       </c>
       <c r="F13" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -6594,13 +6594,13 @@
         <v>154</v>
       </c>
       <c r="D14" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E14" s="4">
         <v>45441</v>
       </c>
       <c r="F14" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -6614,13 +6614,13 @@
         <v>155</v>
       </c>
       <c r="D15" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E15" s="4">
         <v>45492</v>
       </c>
       <c r="F15" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -6634,13 +6634,13 @@
         <v>148</v>
       </c>
       <c r="D16" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E16" s="4">
         <v>45741</v>
       </c>
       <c r="F16" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -6654,13 +6654,13 @@
         <v>156</v>
       </c>
       <c r="D17" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E17" s="4">
         <v>45805</v>
       </c>
       <c r="F17" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -6674,13 +6674,13 @@
         <v>157</v>
       </c>
       <c r="D18" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E18" s="4">
         <v>45805</v>
       </c>
       <c r="F18" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -6691,16 +6691,16 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D19" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E19" s="4">
         <v>45867</v>
       </c>
       <c r="F19" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -6711,16 +6711,16 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D20" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="E20" s="4">
         <v>46108</v>
       </c>
       <c r="F20" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -6731,16 +6731,16 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="D21" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E21" s="4">
         <v>46175</v>
       </c>
       <c r="F21" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -7423,7 +7423,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D2" t="s">
         <v>60</v>
@@ -7446,7 +7446,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D3" t="s">
         <v>59</v>
@@ -7495,7 +7495,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -7510,7 +7510,7 @@
         <v>135</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -7521,10 +7521,10 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="D6" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="E6" s="4">
         <v>46105</v>
@@ -7542,7 +7542,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="D7" t="s">
         <v>42</v>
@@ -7557,7 +7557,7 @@
         <v>135</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -7568,10 +7568,10 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E8" s="4">
         <v>45565</v>
@@ -7591,10 +7591,10 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D9" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E9" s="4">
         <v>45616</v>
@@ -7614,10 +7614,10 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D10" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E10" s="4">
         <v>45565</v>
@@ -7640,7 +7640,7 @@
         <v>129</v>
       </c>
       <c r="D11" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E11" s="4">
         <v>45876</v>
@@ -7649,7 +7649,7 @@
         <v>135</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -7681,7 +7681,7 @@
         <v>131</v>
       </c>
       <c r="D13" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="E13" s="4">
         <v>45871</v>
@@ -7716,10 +7716,10 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="D15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E15" s="4">
         <v>45901</v>
@@ -7729,7 +7729,7 @@
         <v>135</v>
       </c>
       <c r="H15" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -7987,7 +7987,7 @@
         <v>97</v>
       </c>
       <c r="F1" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -8004,7 +8004,7 @@
         <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F2">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8025,7 +8025,7 @@
         <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F3">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8046,7 +8046,7 @@
         <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F4">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8067,7 +8067,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F5">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8088,7 +8088,7 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F6">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8109,7 +8109,7 @@
         <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F7">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8130,7 +8130,7 @@
         <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F8">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8151,7 +8151,7 @@
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F9">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8172,7 +8172,7 @@
         <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F10">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8193,7 +8193,7 @@
         <v>9</v>
       </c>
       <c r="E11" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F11">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8214,7 +8214,7 @@
         <v>6</v>
       </c>
       <c r="E12" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F12">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8235,7 +8235,7 @@
         <v>8</v>
       </c>
       <c r="E13" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="F13">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8256,7 +8256,7 @@
         <v>7</v>
       </c>
       <c r="E14" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F14">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8277,7 +8277,7 @@
         <v>6</v>
       </c>
       <c r="E15" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F15">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8298,7 +8298,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F16">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8319,7 +8319,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="F17">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8340,7 +8340,7 @@
         <v>9</v>
       </c>
       <c r="E18" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F18">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8361,7 +8361,7 @@
         <v>8</v>
       </c>
       <c r="E19" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F19">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8382,7 +8382,7 @@
         <v>8</v>
       </c>
       <c r="E20" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="F20">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8403,7 +8403,7 @@
         <v>7</v>
       </c>
       <c r="E21" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F21">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8424,7 +8424,7 @@
         <v>6</v>
       </c>
       <c r="E22" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F22">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8445,7 +8445,7 @@
         <v>8</v>
       </c>
       <c r="E23" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F23">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8466,7 +8466,7 @@
         <v>7</v>
       </c>
       <c r="E24" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F24">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>
@@ -8478,7 +8478,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C25" s="30" t="s">
         <v>164</v>
@@ -8487,7 +8487,7 @@
         <v>6</v>
       </c>
       <c r="E25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F25">
         <f>COUNTIF(Table8[skill_id],Table412[[#This Row],[skill_id]])</f>

</xml_diff>

<commit_message>
Integrated Paper II Publication into Portfolio Highlights in Researcher Domain
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6C0E84-25E4-5145-8351-58891A775BEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F5D7AB-7017-D741-B810-33D01CB92CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="11" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
+    <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="6" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
   <sheets>
     <sheet name="person" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="300">
   <si>
     <t>Graduation</t>
   </si>
@@ -894,9 +894,6 @@
     <t>https://public.tableau.com/app/profile/cedric.hering.peter/viz/CV-Dashboard_17551211549430/Published_Apr-26?publish=yes</t>
   </si>
   <si>
-    <t>Paper in Bioresource Technology</t>
-  </si>
-  <si>
     <t>Paper in Journal  of Applied Phycology</t>
   </si>
   <si>
@@ -946,6 +943,12 @@
   </si>
   <si>
     <t>fluorescence imaging, z-stack imaging</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1016/j.biortech.2026.135341</t>
+  </si>
+  <si>
+    <t>Paper in Bio-          resource Technology</t>
   </si>
 </sst>
 </file>
@@ -3857,7 +3860,7 @@
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F14">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -3953,7 +3956,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C19" t="s">
         <v>168</v>
@@ -3962,7 +3965,7 @@
         <v>4</v>
       </c>
       <c r="E19" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F19">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -4046,7 +4049,7 @@
         <v>4</v>
       </c>
       <c r="E23" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F23">
         <f>COUNTIF(Table7[tool_id],Table4[[#This Row],[tool_id]])</f>
@@ -5600,7 +5603,7 @@
         <v>158</v>
       </c>
       <c r="D2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E2" t="s">
         <v>159</v>
@@ -5614,7 +5617,7 @@
         <v>2</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -5622,13 +5625,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C4" t="s">
         <v>238</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E4" t="s">
         <v>161</v>
@@ -5639,13 +5642,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C5" t="s">
         <v>237</v>
       </c>
       <c r="D5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="E5" t="s">
         <v>160</v>
@@ -5662,10 +5665,10 @@
         <v>239</v>
       </c>
       <c r="D6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -6691,7 +6694,7 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D19" t="s">
         <v>233</v>
@@ -6731,7 +6734,7 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D21" t="s">
         <v>233</v>
@@ -6740,7 +6743,7 @@
         <v>46175</v>
       </c>
       <c r="F21" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -7495,7 +7498,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
@@ -7521,7 +7524,7 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>281</v>
+        <v>299</v>
       </c>
       <c r="D6" t="s">
         <v>276</v>
@@ -7529,9 +7532,14 @@
       <c r="E6" s="4">
         <v>46105</v>
       </c>
-      <c r="F6" s="4"/>
+      <c r="F6" s="4">
+        <v>46211</v>
+      </c>
       <c r="G6" t="s">
-        <v>136</v>
+        <v>135</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -7542,7 +7550,7 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D7" t="s">
         <v>42</v>
@@ -7645,6 +7653,9 @@
       <c r="E11" s="4">
         <v>45876</v>
       </c>
+      <c r="F11" s="4">
+        <v>46131</v>
+      </c>
       <c r="G11" t="s">
         <v>135</v>
       </c>
@@ -7686,6 +7697,7 @@
       <c r="E13" s="4">
         <v>45871</v>
       </c>
+      <c r="F13" s="4"/>
       <c r="G13" t="s">
         <v>136</v>
       </c>
@@ -7742,11 +7754,12 @@
     <hyperlink ref="H10" r:id="rId5" xr:uid="{C273DA0B-17C9-0F49-AAE4-F1DFD24E4CA4}"/>
     <hyperlink ref="H7" r:id="rId6" xr:uid="{38A82EE0-E664-4B49-9718-B5EF47828CDB}"/>
     <hyperlink ref="H11" r:id="rId7" xr:uid="{160F5AC7-78D1-E347-BC0D-6E1E9E6301BF}"/>
+    <hyperlink ref="H6" r:id="rId8" xr:uid="{FA3D473E-3130-D64F-ADC5-D54F83AE276E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Executed pipeline and fixed formatting issues in the paper description panel
</commit_message>
<xml_diff>
--- a/01_Data/raw/master_database.xlsx
+++ b/01_Data/raw/master_database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cedric/Documents/13_Personal/131_Profile-and-Planning/01_Resume-and-Portfolio/03_Visual-Resume_Tableau-Dashboard/01_Data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F5D7AB-7017-D741-B810-33D01CB92CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E96409-C800-0349-BEEE-220968F245C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="680" yWindow="600" windowWidth="50520" windowHeight="28200" activeTab="6" xr2:uid="{52660A98-60EA-894E-A12F-88F737DC9EAD}"/>
   </bookViews>
@@ -948,7 +948,7 @@
     <t>https://doi.org/10.1016/j.biortech.2026.135341</t>
   </si>
   <si>
-    <t>Paper in Bio-          resource Technology</t>
+    <t>Paper in Biore-   source Technology</t>
   </si>
 </sst>
 </file>
@@ -1326,12 +1326,6 @@
       </border>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1368,6 +1362,12 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
@@ -1506,8 +1506,8 @@
     <tableColumn id="3" xr3:uid="{519CB3FD-482A-2B44-9C5A-9E797E3F98E4}" name="title"/>
     <tableColumn id="4" xr3:uid="{0DBFEBFC-D18A-6F4E-87F2-C8D4D16C7E2D}" name="organization"/>
     <tableColumn id="9" xr3:uid="{3E657E01-C34B-0B41-8B45-85D9AE50305B}" name="location"/>
-    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{0E638BC4-2710-0C43-A1C1-191B65B559E5}" name="start_date" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{B967E793-1F53-A448-B344-EC57AFC8844D}" name="end_date" dataDxfId="6"/>
     <tableColumn id="8" xr3:uid="{4B60B559-FFE2-0449-BD87-E423F2579CE2}" name="description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1518,7 +1518,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}" name="Table14" displayName="Table14" ref="A1:B24" totalsRowShown="0">
   <autoFilter ref="A1:B24" xr:uid="{9EDB993D-0CDD-3346-B634-A5B977627571}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{D1FF01A2-FC84-1441-97CB-D234B9FA64EA}" name="activity_id" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{647E29E8-3B30-6747-952B-856B15C586DD}" name="domain_id"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1559,8 +1559,8 @@
     <tableColumn id="6" xr3:uid="{D37906CD-C2EB-8A40-AA51-891ADDD2F0F3}" name="person_id"/>
     <tableColumn id="8" xr3:uid="{912FC1CE-8929-A840-BCE1-17117B008FD3}" name="title"/>
     <tableColumn id="11" xr3:uid="{8675359A-ECB9-7944-B6E4-F8EFBA93E841}" name="description"/>
-    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="6"/>
-    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{CA3124FD-9F98-C74D-B3D4-70469E4BA6CD}" name="start_date" dataDxfId="9"/>
+    <tableColumn id="14" xr3:uid="{B8D40936-6AA7-A74A-ACA0-517CCCC4CB7F}" name="end_date" dataDxfId="8"/>
     <tableColumn id="1" xr3:uid="{D859FDAD-79F9-EC41-ACD6-64B4107CA00A}" name="status"/>
     <tableColumn id="12" xr3:uid="{267EBF1D-F600-6746-8520-55E6EE075513}" name="link"/>
   </tableColumns>

</xml_diff>